<commit_message>
Add uranium data for 34 J22 samples from ZU23_09to10M
Data sourced from Results_U236_Mar2023_JOIS22_TA_ZU23_09to10M.xlsx.
Fills U238_ppb, unc_U238_ppb, U236_U238, unc_U236_U238 for samples
J22 25-47, 196-315 range.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00_j22_isotopes.xlsx
+++ b/00_j22_isotopes.xlsx
@@ -669,6 +669,18 @@
       <c r="Y2" t="n">
         <v>1.042006714500043</v>
       </c>
+      <c r="AB2" t="n">
+        <v>2.64626862883549</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0.03969402943253236</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1411.638474926253</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>33.75493168598892</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -762,6 +774,18 @@
       <c r="AA3" t="n">
         <v>0.2413220983083535</v>
       </c>
+      <c r="AB3" t="n">
+        <v>3.033022178875957</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.05956248789646976</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1347.829249616784</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>40.51487826441279</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -855,6 +879,18 @@
       <c r="AA4" t="n">
         <v>0.2963662532099018</v>
       </c>
+      <c r="AB4" t="n">
+        <v>3.15330338956795</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0.05782221889752515</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1703.18280475709</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>47.80054962483911</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -948,6 +984,18 @@
       <c r="AA5" t="n">
         <v>0.2917383477196132</v>
       </c>
+      <c r="AB5" t="n">
+        <v>3.175980111297348</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.06472078695449644</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1863.987665303361</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>51.89414159940792</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1041,6 +1089,18 @@
       <c r="AA6" t="n">
         <v>0.484238950415394</v>
       </c>
+      <c r="AB6" t="n">
+        <v>3.439515291393985</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0.05906415348850569</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>3230.185069914932</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>77.50565694227869</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1134,6 +1194,18 @@
       <c r="AA7" t="n">
         <v>0.614039118821314</v>
       </c>
+      <c r="AB7" t="n">
+        <v>3.309044101716357</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0.05746829810411269</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>3208.552288397774</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>90.52871122953241</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1227,6 +1299,18 @@
       <c r="AA8" t="n">
         <v>0.4851716442708776</v>
       </c>
+      <c r="AB8" t="n">
+        <v>3.284711617649038</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0.04927067426473557</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>3268.766614316724</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>75.02780038965159</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1320,6 +1404,18 @@
       <c r="AA9" t="n">
         <v>0.5302653581813255</v>
       </c>
+      <c r="AB9" t="n">
+        <v>3.249670701638879</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0.04874506052458318</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>3226.029971686591</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>79.23115498613573</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6483,6 +6579,18 @@
       <c r="AA59" t="n">
         <v>0.1566052472970075</v>
       </c>
+      <c r="AB59" t="n">
+        <v>2.556234400793072</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>0.0390351573406285</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>1283.924361101145</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>30.77309805022378</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6576,6 +6684,18 @@
       <c r="AA60" t="n">
         <v>0.1937383832156183</v>
       </c>
+      <c r="AB60" t="n">
+        <v>2.995348563588413</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>0.05850291426384479</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>1117.335171397997</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>33.13836721576664</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6669,6 +6789,18 @@
       <c r="AA61" t="n">
         <v>0.1738454530350423</v>
       </c>
+      <c r="AB61" t="n">
+        <v>2.996649022544409</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>0.04790318575662179</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>1056.3911260799</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>28.01568714537315</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6762,6 +6894,18 @@
       <c r="AA62" t="n">
         <v>0.2451029001112112</v>
       </c>
+      <c r="AB62" t="n">
+        <v>3.14238487499351</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>0.04713577312490266</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>1415.441561940191</v>
+      </c>
+      <c r="AE62" t="n">
+        <v>36.77334618699173</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6855,6 +6999,18 @@
       <c r="AA63" t="n">
         <v>0.5169037719815656</v>
       </c>
+      <c r="AB63" t="n">
+        <v>3.207492941064758</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>0.04811239411597137</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>3232.954249656746</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>78.69198519394585</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6948,6 +7104,18 @@
       <c r="AA64" t="n">
         <v>0.5919512982962961</v>
       </c>
+      <c r="AB64" t="n">
+        <v>3.131543793839339</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>0.04697315690759008</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>2943.564853567602</v>
+      </c>
+      <c r="AE64" t="n">
+        <v>85.03979040956051</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7041,6 +7209,18 @@
       <c r="AA65" t="n">
         <v>0.3877696265404994</v>
       </c>
+      <c r="AB65" t="n">
+        <v>3.265296699000105</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>0.05931850859250404</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>2521.14174581828</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>64.66941282287432</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7134,6 +7314,18 @@
       <c r="AA66" t="n">
         <v>0.3888601315708009</v>
       </c>
+      <c r="AB66" t="n">
+        <v>3.289749378808673</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>0.06692692690142427</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>2593.102900529951</v>
+      </c>
+      <c r="AE66" t="n">
+        <v>69.62839459763377</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7227,6 +7419,18 @@
       <c r="AA67" t="n">
         <v>0.406242333895467</v>
       </c>
+      <c r="AB67" t="n">
+        <v>3.283676185099668</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>0.05134578280013585</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>2369.394782648866</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>60.28861647004713</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7320,6 +7524,18 @@
       <c r="AA68" t="n">
         <v>0.3643640719687847</v>
       </c>
+      <c r="AB68" t="n">
+        <v>3.340830341713371</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>0.05011245512570057</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>2282.185098964082</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>54.12755228993998</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7413,6 +7629,18 @@
       <c r="AA69" t="n">
         <v>0.2480252948931392</v>
       </c>
+      <c r="AB69" t="n">
+        <v>3.362399797463641</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>0.06317752530126897</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>1073.801286098606</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>34.80139731902036</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7506,6 +7734,18 @@
       <c r="AA70" t="n">
         <v>0.1066167277180454</v>
       </c>
+      <c r="AB70" t="n">
+        <v>3.3470577121664</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>0.06274460352543894</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>225.0467676927616</v>
+      </c>
+      <c r="AE70" t="n">
+        <v>12.95106413137865</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7599,6 +7839,18 @@
       <c r="AA71" t="n">
         <v>0.01306931813756102</v>
       </c>
+      <c r="AB71" t="n">
+        <v>3.205379399895319</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>0.0589209826502298</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>7.366155426861447</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>1.573141397605726</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10368,6 +10620,18 @@
       <c r="AA98" t="n">
         <v>0.1932526723626782</v>
       </c>
+      <c r="AB98" t="n">
+        <v>2.358978703435412</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>0.03981581416245366</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>1429.290318563854</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>39.8634810008002</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10461,6 +10725,18 @@
       <c r="AA99" t="n">
         <v>0.2304150722147032</v>
       </c>
+      <c r="AB99" t="n">
+        <v>3.003779889991435</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>0.05419626471429651</v>
+      </c>
+      <c r="AD99" t="n">
+        <v>1125.473593839603</v>
+      </c>
+      <c r="AE99" t="n">
+        <v>35.88200919118415</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -10554,6 +10830,18 @@
       <c r="AA100" t="n">
         <v>0.1720923748347519</v>
       </c>
+      <c r="AB100" t="n">
+        <v>2.953715321867236</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>0.04430572982800855</v>
+      </c>
+      <c r="AD100" t="n">
+        <v>1064.382797069761</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>27.54932745065245</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10647,6 +10935,18 @@
       <c r="AA101" t="n">
         <v>0.4061627726102852</v>
       </c>
+      <c r="AB101" t="n">
+        <v>3.199845578766583</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>0.04958247146545475</v>
+      </c>
+      <c r="AD101" t="n">
+        <v>1493.379815612966</v>
+      </c>
+      <c r="AE101" t="n">
+        <v>54.06275631295034</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -10740,6 +11040,18 @@
       <c r="AA102" t="n">
         <v>0.7014851248789741</v>
       </c>
+      <c r="AB102" t="n">
+        <v>3.313749630113928</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>0.05568267470236377</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>3521.504368303802</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>100.6405603088197</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10833,6 +11145,18 @@
       <c r="AA103" t="n">
         <v>0.6621904833365152</v>
       </c>
+      <c r="AB103" t="n">
+        <v>3.503938103632354</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>0.06397608674524521</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>3019.037583768577</v>
+      </c>
+      <c r="AE103" t="n">
+        <v>91.20481437137592</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10926,6 +11250,18 @@
       <c r="AA104" t="n">
         <v>0.4843324499058317</v>
       </c>
+      <c r="AB104" t="n">
+        <v>3.240917294221978</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>0.04861375941332967</v>
+      </c>
+      <c r="AD104" t="n">
+        <v>2799.253166847052</v>
+      </c>
+      <c r="AE104" t="n">
+        <v>71.16253087391155</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -11019,6 +11355,18 @@
       <c r="AA105" t="n">
         <v>0.4587664934834027</v>
       </c>
+      <c r="AB105" t="n">
+        <v>3.243762650647426</v>
+      </c>
+      <c r="AC105" t="n">
+        <v>0.05048651016045202</v>
+      </c>
+      <c r="AD105" t="n">
+        <v>2751.228188215642</v>
+      </c>
+      <c r="AE105" t="n">
+        <v>69.21005005877491</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11112,6 +11460,18 @@
       <c r="AA106" t="n">
         <v>0.4721244218477029</v>
       </c>
+      <c r="AB106" t="n">
+        <v>3.362823679831733</v>
+      </c>
+      <c r="AC106" t="n">
+        <v>0.06447795334643525</v>
+      </c>
+      <c r="AD106" t="n">
+        <v>2553.949421655148</v>
+      </c>
+      <c r="AE106" t="n">
+        <v>72.87710048400072</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11205,6 +11565,18 @@
       <c r="AA107" t="n">
         <v>0.4391355328992175</v>
       </c>
+      <c r="AB107" t="n">
+        <v>3.151501444875708</v>
+      </c>
+      <c r="AC107" t="n">
+        <v>0.05170772912849702</v>
+      </c>
+      <c r="AD107" t="n">
+        <v>2575.010647733152</v>
+      </c>
+      <c r="AE107" t="n">
+        <v>68.22332087024452</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11298,6 +11670,18 @@
       <c r="AA108" t="n">
         <v>0.2610676714320252</v>
       </c>
+      <c r="AB108" t="n">
+        <v>3.430085309529745</v>
+      </c>
+      <c r="AC108" t="n">
+        <v>0.06221362503612025</v>
+      </c>
+      <c r="AD108" t="n">
+        <v>1072.106798267212</v>
+      </c>
+      <c r="AE108" t="n">
+        <v>35.13065045808858</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11391,6 +11775,18 @@
       <c r="AA109" t="n">
         <v>0.07037325509247865</v>
       </c>
+      <c r="AB109" t="n">
+        <v>3.395516528288801</v>
+      </c>
+      <c r="AC109" t="n">
+        <v>0.07176158725136531</v>
+      </c>
+      <c r="AD109" t="n">
+        <v>228.097317676254</v>
+      </c>
+      <c r="AE109" t="n">
+        <v>9.311790741480761</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -11483,6 +11879,18 @@
       </c>
       <c r="AA110" t="n">
         <v>0.008994188551172792</v>
+      </c>
+      <c r="AB110" t="n">
+        <v>3.325587222554091</v>
+      </c>
+      <c r="AC110" t="n">
+        <v>0.05804216910829469</v>
+      </c>
+      <c r="AD110" t="n">
+        <v>4.68860250473508</v>
+      </c>
+      <c r="AE110" t="n">
+        <v>1.042831745976585</v>
       </c>
     </row>
     <row r="111">

</xml_diff>

<commit_message>
Reformat isotope file to uniform schema with TEOS-10 derived variables
Standardise column order and headers. Rename Salinity -> Salinity_psu.
Compute Conservative_Temp, Potential_Temp, and Absolute_Salinity using
gsw (TEOS-10). Populate uranium columns (U238_ppb, U236_U238, etc.)
from AMS measurement files.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00_j22_isotopes.xlsx
+++ b/00_j22_isotopes.xlsx
@@ -603,9 +603,18 @@
       <c r="J2" t="n">
         <v>3.2875</v>
       </c>
+      <c r="K2" t="n">
+        <v>3.344987201039375</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3.287205005978202</v>
+      </c>
       <c r="M2" t="n">
         <v>27.6802</v>
       </c>
+      <c r="N2" t="n">
+        <v>27.81340284954568</v>
+      </c>
       <c r="O2" t="n">
         <v>22.03565560347351</v>
       </c>
@@ -683,9 +692,18 @@
       <c r="J3" t="n">
         <v>-1.049</v>
       </c>
+      <c r="K3" t="n">
+        <v>-1.039278189314062</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-1.049604943265887</v>
+      </c>
       <c r="M3" t="n">
         <v>31.2421</v>
       </c>
+      <c r="N3" t="n">
+        <v>31.39334471108419</v>
+      </c>
       <c r="O3" t="n">
         <v>25.11682364604371</v>
       </c>
@@ -769,9 +787,18 @@
       <c r="J4" t="n">
         <v>-1.1744</v>
       </c>
+      <c r="K4" t="n">
+        <v>-1.169932556338563</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-1.176610784283774</v>
+      </c>
       <c r="M4" t="n">
         <v>32.8468</v>
       </c>
+      <c r="N4" t="n">
+        <v>33.00977358837617</v>
+      </c>
       <c r="O4" t="n">
         <v>26.42257870075628</v>
       </c>
@@ -855,9 +882,18 @@
       <c r="J5" t="n">
         <v>-1.0952</v>
       </c>
+      <c r="K5" t="n">
+        <v>-1.092127559245875</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-1.098122476988568</v>
+      </c>
       <c r="M5" t="n">
         <v>33.2132</v>
       </c>
+      <c r="N5" t="n">
+        <v>33.37811737077585</v>
+      </c>
       <c r="O5" t="n">
         <v>26.7108395076873</v>
       </c>
@@ -941,9 +977,18 @@
       <c r="J6" t="n">
         <v>0.2942</v>
       </c>
+      <c r="K6" t="n">
+        <v>0.2830028980877877</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2818873383836472</v>
+      </c>
       <c r="M6" t="n">
         <v>34.6833</v>
       </c>
+      <c r="N6" t="n">
+        <v>34.85070804994395</v>
+      </c>
       <c r="O6" t="n">
         <v>27.8388329892116</v>
       </c>
@@ -1027,9 +1072,18 @@
       <c r="J7" t="n">
         <v>0.3477</v>
       </c>
+      <c r="K7" t="n">
+        <v>0.3339830000249136</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.3330570800148892</v>
+      </c>
       <c r="M7" t="n">
         <v>34.7131</v>
       </c>
+      <c r="N7" t="n">
+        <v>34.8806985462611</v>
+      </c>
       <c r="O7" t="n">
         <v>27.85973096677253</v>
       </c>
@@ -1113,9 +1167,18 @@
       <c r="J8" t="n">
         <v>0.4225</v>
       </c>
+      <c r="K8" t="n">
+        <v>0.4014152215143384</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.4007184722080885</v>
+      </c>
       <c r="M8" t="n">
         <v>34.7472</v>
       </c>
+      <c r="N8" t="n">
+        <v>34.91448925638008</v>
+      </c>
       <c r="O8" t="n">
         <v>27.8827618089224</v>
       </c>
@@ -1199,9 +1262,18 @@
       <c r="J9" t="n">
         <v>0.4497</v>
       </c>
+      <c r="K9" t="n">
+        <v>0.4239111638697245</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.4232723927446225</v>
+      </c>
       <c r="M9" t="n">
         <v>34.7544</v>
       </c>
+      <c r="N9" t="n">
+        <v>34.92172392054427</v>
+      </c>
       <c r="O9" t="n">
         <v>27.88733114088404</v>
       </c>
@@ -1285,9 +1357,18 @@
       <c r="J10" t="n">
         <v>-0.8615</v>
       </c>
+      <c r="K10" t="n">
+        <v>-0.8483607771245213</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-0.8616145141268354</v>
+      </c>
       <c r="M10" t="n">
         <v>30.2406</v>
       </c>
+      <c r="N10" t="n">
+        <v>30.38573667584751</v>
+      </c>
       <c r="O10" t="n">
         <v>24.29902215574793</v>
       </c>
@@ -1371,9 +1452,18 @@
       <c r="J11" t="n">
         <v>-0.8633</v>
       </c>
+      <c r="K11" t="n">
+        <v>-0.8501730405997576</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-0.8634178299656806</v>
+      </c>
       <c r="M11" t="n">
         <v>30.2397</v>
       </c>
+      <c r="N11" t="n">
+        <v>30.38482517980696</v>
+      </c>
       <c r="O11" t="n">
         <v>24.29986482991126</v>
       </c>
@@ -1457,9 +1547,18 @@
       <c r="J12" t="n">
         <v>-0.5816</v>
       </c>
+      <c r="K12" t="n">
+        <v>-0.5705811829521612</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-0.5824579398980794</v>
+      </c>
       <c r="M12" t="n">
         <v>31.431</v>
       </c>
+      <c r="N12" t="n">
+        <v>31.58217017056593</v>
+      </c>
       <c r="O12" t="n">
         <v>25.2679045050802</v>
       </c>
@@ -1543,9 +1642,18 @@
       <c r="J13" t="n">
         <v>-1.207</v>
       </c>
+      <c r="K13" t="n">
+        <v>-1.204524887701752</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-1.21050739424183</v>
+      </c>
       <c r="M13" t="n">
         <v>33.1483</v>
       </c>
+      <c r="N13" t="n">
+        <v>33.311614406783</v>
+      </c>
       <c r="O13" t="n">
         <v>26.66927832858119</v>
       </c>
@@ -1629,9 +1737,18 @@
       <c r="J14" t="n">
         <v>-0.1863</v>
       </c>
+      <c r="K14" t="n">
+        <v>-0.192023965785023</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.1945559644959328</v>
+      </c>
       <c r="M14" t="n">
         <v>34.435</v>
       </c>
+      <c r="N14" t="n">
+        <v>34.60180315737149</v>
+      </c>
       <c r="O14" t="n">
         <v>27.66025900012596</v>
       </c>
@@ -1691,9 +1808,18 @@
       <c r="J15" t="n">
         <v>0.4056</v>
       </c>
+      <c r="K15" t="n">
+        <v>0.3938825689244529</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.3929783272942971</v>
+      </c>
       <c r="M15" t="n">
         <v>34.7062</v>
       </c>
+      <c r="N15" t="n">
+        <v>34.87373182297194</v>
+      </c>
       <c r="O15" t="n">
         <v>27.85037514348915</v>
       </c>
@@ -1777,9 +1903,18 @@
       <c r="J16" t="n">
         <v>0.708</v>
       </c>
+      <c r="K16" t="n">
+        <v>0.6898750005508781</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.6897193157306215</v>
+      </c>
       <c r="M16" t="n">
         <v>34.7949</v>
       </c>
+      <c r="N16" t="n">
+        <v>34.96266684080356</v>
+      </c>
       <c r="O16" t="n">
         <v>27.90347663275156</v>
       </c>
@@ -1839,9 +1974,18 @@
       <c r="J17" t="n">
         <v>0.7677</v>
       </c>
+      <c r="K17" t="n">
+        <v>0.7386379470903831</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.7388928865484982</v>
+      </c>
       <c r="M17" t="n">
         <v>34.8612</v>
       </c>
+      <c r="N17" t="n">
+        <v>35.02868366693684</v>
+      </c>
       <c r="O17" t="n">
         <v>27.95311052275815</v>
       </c>
@@ -1925,9 +2069,18 @@
       <c r="J18" t="n">
         <v>0.459</v>
       </c>
+      <c r="K18" t="n">
+        <v>0.4213160077166296</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.4212499792614479</v>
+      </c>
       <c r="M18" t="n">
         <v>34.87</v>
       </c>
+      <c r="N18" t="n">
+        <v>35.03747261187637</v>
+      </c>
       <c r="O18" t="n">
         <v>27.97980272405698</v>
       </c>
@@ -2011,9 +2164,18 @@
       <c r="J19" t="n">
         <v>-0.0727</v>
       </c>
+      <c r="K19" t="n">
+        <v>-0.1247662762799567</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-0.1253796800572646</v>
+      </c>
       <c r="M19" t="n">
         <v>34.8914</v>
       </c>
+      <c r="N19" t="n">
+        <v>35.05902840816285</v>
+      </c>
       <c r="O19" t="n">
         <v>28.02764671480622</v>
       </c>
@@ -2097,9 +2259,18 @@
       <c r="J20" t="n">
         <v>-0.3142</v>
       </c>
+      <c r="K20" t="n">
+        <v>-0.2957026295352292</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-0.3143169403851928</v>
+      </c>
       <c r="M20" t="n">
         <v>29.4647</v>
       </c>
+      <c r="N20" t="n">
+        <v>29.60615612165097</v>
+      </c>
       <c r="O20" t="n">
         <v>23.65593916546754</v>
       </c>
@@ -2183,9 +2354,18 @@
       <c r="J21" t="n">
         <v>-0.0506</v>
       </c>
+      <c r="K21" t="n">
+        <v>-0.03577302122348491</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-0.05157971557179165</v>
+      </c>
       <c r="M21" t="n">
         <v>30.9158</v>
       </c>
+      <c r="N21" t="n">
+        <v>31.06446250782385</v>
+      </c>
       <c r="O21" t="n">
         <v>24.81749453456177</v>
       </c>
@@ -2269,9 +2449,18 @@
       <c r="J22" t="n">
         <v>-0.2421</v>
       </c>
+      <c r="K22" t="n">
+        <v>-0.2317659527561412</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-0.2436377603066601</v>
+      </c>
       <c r="M22" t="n">
         <v>31.8549</v>
       </c>
+      <c r="N22" t="n">
+        <v>32.00841166002422</v>
+      </c>
       <c r="O22" t="n">
         <v>25.58924236938674</v>
       </c>
@@ -2355,9 +2544,18 @@
       <c r="J23" t="n">
         <v>-1.1938</v>
       </c>
+      <c r="K23" t="n">
+        <v>-1.191348699459718</v>
+      </c>
+      <c r="L23" t="n">
+        <v>-1.197224517386896</v>
+      </c>
       <c r="M23" t="n">
         <v>33.207</v>
       </c>
+      <c r="N23" t="n">
+        <v>33.37034017088989</v>
+      </c>
       <c r="O23" t="n">
         <v>26.7103940043628</v>
       </c>
@@ -2441,9 +2639,18 @@
       <c r="J24" t="n">
         <v>-0.2152</v>
       </c>
+      <c r="K24" t="n">
+        <v>-0.2205331051931673</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-0.2231204073298678</v>
+      </c>
       <c r="M24" t="n">
         <v>34.4245</v>
       </c>
+      <c r="N24" t="n">
+        <v>34.59144170215679</v>
+      </c>
       <c r="O24" t="n">
         <v>27.65589491709716</v>
       </c>
@@ -2527,9 +2734,18 @@
       <c r="J25" t="n">
         <v>0.3532</v>
       </c>
+      <c r="K25" t="n">
+        <v>0.3424217895341167</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.3414334197374956</v>
+      </c>
       <c r="M25" t="n">
         <v>34.6985</v>
       </c>
+      <c r="N25" t="n">
+        <v>34.8661331413515</v>
+      </c>
       <c r="O25" t="n">
         <v>27.84701896706656</v>
       </c>
@@ -2613,9 +2829,18 @@
       <c r="J26" t="n">
         <v>0.8241000000000001</v>
       </c>
+      <c r="K26" t="n">
+        <v>0.8018807914321278</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.8021407012026525</v>
+      </c>
       <c r="M26" t="n">
         <v>34.8485</v>
       </c>
+      <c r="N26" t="n">
+        <v>35.01650722313398</v>
+      </c>
       <c r="O26" t="n">
         <v>27.93915892945142</v>
       </c>
@@ -2699,9 +2924,18 @@
       <c r="J27" t="n">
         <v>0.6771</v>
       </c>
+      <c r="K27" t="n">
+        <v>0.648660699315303</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.6488157621385329</v>
+      </c>
       <c r="M27" t="n">
         <v>34.8618</v>
       </c>
+      <c r="N27" t="n">
+        <v>35.02931977943253</v>
+      </c>
       <c r="O27" t="n">
         <v>27.95917679796867</v>
       </c>
@@ -2785,9 +3019,18 @@
       <c r="J28" t="n">
         <v>0.422</v>
       </c>
+      <c r="K28" t="n">
+        <v>0.3847112515300838</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.3846060633798506</v>
+      </c>
       <c r="M28" t="n">
         <v>34.8707</v>
       </c>
+      <c r="N28" t="n">
+        <v>35.03818044387055</v>
+      </c>
       <c r="O28" t="n">
         <v>27.98229615555374</v>
       </c>
@@ -2871,9 +3114,18 @@
       <c r="J29" t="n">
         <v>-0.011</v>
       </c>
+      <c r="K29" t="n">
+        <v>-0.0554089844837537</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-0.05595873150424029</v>
+      </c>
       <c r="M29" t="n">
         <v>34.8869</v>
       </c>
+      <c r="N29" t="n">
+        <v>35.05444944388098</v>
+      </c>
       <c r="O29" t="n">
         <v>28.02016709330383</v>
       </c>
@@ -2957,9 +3209,18 @@
       <c r="J30" t="n">
         <v>-0.3388</v>
       </c>
+      <c r="K30" t="n">
+        <v>-0.4081336688497527</v>
+      </c>
+      <c r="L30" t="n">
+        <v>-0.4089768028144348</v>
+      </c>
       <c r="M30" t="n">
         <v>34.9201</v>
       </c>
+      <c r="N30" t="n">
+        <v>35.08839871270833</v>
+      </c>
       <c r="O30" t="n">
         <v>28.06528569049965</v>
       </c>
@@ -3043,9 +3304,18 @@
       <c r="J31" t="n">
         <v>-0.3997</v>
       </c>
+      <c r="K31" t="n">
+        <v>-0.5006723661422708</v>
+      </c>
+      <c r="L31" t="n">
+        <v>-0.501542144299528</v>
+      </c>
       <c r="M31" t="n">
         <v>34.9441</v>
       </c>
+      <c r="N31" t="n">
+        <v>35.1127961371327</v>
+      </c>
       <c r="O31" t="n">
         <v>28.0894014704686</v>
       </c>
@@ -3129,9 +3399,18 @@
       <c r="J32" t="n">
         <v>-0.3213</v>
       </c>
+      <c r="K32" t="n">
+        <v>-0.4985695426625228</v>
+      </c>
+      <c r="L32" t="n">
+        <v>-0.4993802623530296</v>
+      </c>
       <c r="M32" t="n">
         <v>34.9595</v>
       </c>
+      <c r="N32" t="n">
+        <v>35.12832672290116</v>
+      </c>
       <c r="O32" t="n">
         <v>28.10175160416952</v>
       </c>
@@ -3215,9 +3494,18 @@
       <c r="J33" t="n">
         <v>-1.4778</v>
       </c>
+      <c r="K33" t="n">
+        <v>-1.46646397208533</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-1.477838647961958</v>
+      </c>
       <c r="M33" t="n">
         <v>27.5739</v>
       </c>
+      <c r="N33" t="n">
+        <v>27.70678863104775</v>
+      </c>
       <c r="O33" t="n">
         <v>22.15196088245273</v>
       </c>
@@ -3301,9 +3589,18 @@
       <c r="J34" t="n">
         <v>-0.9264</v>
       </c>
+      <c r="K34" t="n">
+        <v>-0.91637226292317</v>
+      </c>
+      <c r="L34" t="n">
+        <v>-0.9272628076289813</v>
+      </c>
       <c r="M34" t="n">
         <v>31.2307</v>
       </c>
+      <c r="N34" t="n">
+        <v>31.38162922255632</v>
+      </c>
       <c r="O34" t="n">
         <v>25.10157739277111</v>
       </c>
@@ -3363,9 +3660,18 @@
       <c r="J35" t="n">
         <v>-1.4003</v>
       </c>
+      <c r="K35" t="n">
+        <v>-1.393472413463828</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-1.401333979728778</v>
+      </c>
       <c r="M35" t="n">
         <v>31.8668</v>
       </c>
+      <c r="N35" t="n">
+        <v>32.0211634119119</v>
+      </c>
       <c r="O35" t="n">
         <v>25.63328428775867</v>
       </c>
@@ -3449,9 +3755,18 @@
       <c r="J36" t="n">
         <v>-1.4512</v>
       </c>
+      <c r="K36" t="n">
+        <v>-1.448705494322742</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-1.454293340391379</v>
+      </c>
       <c r="M36" t="n">
         <v>33.1653</v>
       </c>
+      <c r="N36" t="n">
+        <v>33.33022239695634</v>
+      </c>
       <c r="O36" t="n">
         <v>26.69281563999311</v>
       </c>
@@ -3532,9 +3847,18 @@
       <c r="J37" t="n">
         <v>-0.7144</v>
       </c>
+      <c r="K37" t="n">
+        <v>-0.7184556415505274</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-0.7212951137074809</v>
+      </c>
       <c r="M37" t="n">
         <v>34.4223</v>
       </c>
+      <c r="N37" t="n">
+        <v>34.58965195707096</v>
+      </c>
       <c r="O37" t="n">
         <v>27.67921157595606</v>
       </c>
@@ -3618,9 +3942,18 @@
       <c r="J38" t="n">
         <v>0.4488</v>
       </c>
+      <c r="K38" t="n">
+        <v>0.4374114507343163</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.4366102440591745</v>
+      </c>
       <c r="M38" t="n">
         <v>34.719</v>
       </c>
+      <c r="N38" t="n">
+        <v>34.88638942277254</v>
+      </c>
       <c r="O38" t="n">
         <v>27.85758604836542</v>
       </c>
@@ -3704,9 +4037,18 @@
       <c r="J39" t="n">
         <v>0.9123</v>
       </c>
+      <c r="K39" t="n">
+        <v>0.8911099830314141</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.8914708914049401</v>
+      </c>
       <c r="M39" t="n">
         <v>34.8489</v>
       </c>
+      <c r="N39" t="n">
+        <v>35.01659200817902</v>
+      </c>
       <c r="O39" t="n">
         <v>27.93346810481466</v>
       </c>
@@ -3790,9 +4132,18 @@
       <c r="J40" t="n">
         <v>0.7514999999999999</v>
       </c>
+      <c r="K40" t="n">
+        <v>0.7224637619069511</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.7227595355724946</v>
+      </c>
       <c r="M40" t="n">
         <v>34.8721</v>
       </c>
+      <c r="N40" t="n">
+        <v>35.03962027854561</v>
+      </c>
       <c r="O40" t="n">
         <v>27.96290187703266</v>
       </c>
@@ -3876,9 +4227,18 @@
       <c r="J41" t="n">
         <v>0.3802</v>
       </c>
+      <c r="K41" t="n">
+        <v>0.3430778166208037</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.3429781629190181</v>
+      </c>
       <c r="M41" t="n">
         <v>34.8819</v>
       </c>
+      <c r="N41" t="n">
+        <v>35.04929181513733</v>
+      </c>
       <c r="O41" t="n">
         <v>27.99387318716913</v>
       </c>
@@ -3962,9 +4322,18 @@
       <c r="J42" t="n">
         <v>0.1027</v>
       </c>
+      <c r="K42" t="n">
+        <v>0.05713228723501071</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.05672367473083994</v>
+      </c>
       <c r="M42" t="n">
         <v>34.8886</v>
       </c>
+      <c r="N42" t="n">
+        <v>35.05598762934905</v>
+      </c>
       <c r="O42" t="n">
         <v>28.01531765346795</v>
       </c>
@@ -4048,9 +4417,18 @@
       <c r="J43" t="n">
         <v>-0.2933</v>
       </c>
+      <c r="K43" t="n">
+        <v>-0.36337823442541</v>
+      </c>
+      <c r="L43" t="n">
+        <v>-0.3641958031462608</v>
+      </c>
       <c r="M43" t="n">
         <v>34.9125</v>
       </c>
+      <c r="N43" t="n">
+        <v>35.08053277147564</v>
+      </c>
       <c r="O43" t="n">
         <v>28.05681598830938</v>
       </c>
@@ -4134,9 +4512,18 @@
       <c r="J44" t="n">
         <v>-0.3997</v>
       </c>
+      <c r="K44" t="n">
+        <v>-0.5008020857323889</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-0.5016679177025417</v>
+      </c>
       <c r="M44" t="n">
         <v>34.9452</v>
       </c>
+      <c r="N44" t="n">
+        <v>35.11393068060734</v>
+      </c>
       <c r="O44" t="n">
         <v>28.09040095623618</v>
       </c>
@@ -4220,9 +4607,18 @@
       <c r="J45" t="n">
         <v>-0.3731</v>
       </c>
+      <c r="K45" t="n">
+        <v>-0.5039564194228352</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-0.5047885306224091</v>
+      </c>
       <c r="M45" t="n">
         <v>34.9554</v>
       </c>
+      <c r="N45" t="n">
+        <v>35.12435855003014</v>
+      </c>
       <c r="O45" t="n">
         <v>28.09881411531342</v>
       </c>
@@ -4306,9 +4702,18 @@
       <c r="J46" t="n">
         <v>-1.4046</v>
       </c>
+      <c r="K46" t="n">
+        <v>-1.392181005298762</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-1.404634550994246</v>
+      </c>
       <c r="M46" t="n">
         <v>26.638</v>
       </c>
+      <c r="N46" t="n">
+        <v>26.76627139883545</v>
+      </c>
       <c r="O46" t="n">
         <v>21.39145662557667</v>
       </c>
@@ -4392,9 +4797,18 @@
       <c r="J47" t="n">
         <v>0.4882</v>
       </c>
+      <c r="K47" t="n">
+        <v>0.5039879634192516</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.4866142084784327</v>
+      </c>
       <c r="M47" t="n">
         <v>31.1562</v>
       </c>
+      <c r="N47" t="n">
+        <v>31.30687916997361</v>
+      </c>
       <c r="O47" t="n">
         <v>24.99969640890095</v>
       </c>
@@ -4478,9 +4892,18 @@
       <c r="J48" t="n">
         <v>-0.6234</v>
       </c>
+      <c r="K48" t="n">
+        <v>-0.6147946660920086</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-0.6252761483554228</v>
+      </c>
       <c r="M48" t="n">
         <v>31.8855</v>
       </c>
+      <c r="N48" t="n">
+        <v>32.04023802825738</v>
+      </c>
       <c r="O48" t="n">
         <v>25.62753969028722</v>
       </c>
@@ -4564,9 +4987,18 @@
       <c r="J49" t="n">
         <v>-1.4691</v>
       </c>
+      <c r="K49" t="n">
+        <v>-1.467138946918582</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-1.472747790697525</v>
+      </c>
       <c r="M49" t="n">
         <v>33.1394</v>
       </c>
+      <c r="N49" t="n">
+        <v>33.30232713660325</v>
+      </c>
       <c r="O49" t="n">
         <v>26.67014207279612</v>
       </c>
@@ -4650,9 +5082,18 @@
       <c r="J50" t="n">
         <v>-0.4029</v>
       </c>
+      <c r="K50" t="n">
+        <v>-0.408851269601115</v>
+      </c>
+      <c r="L50" t="n">
+        <v>-0.4115460987405697</v>
+      </c>
       <c r="M50" t="n">
         <v>34.4213</v>
       </c>
+      <c r="N50" t="n">
+        <v>34.58765567992853</v>
+      </c>
       <c r="O50" t="n">
         <v>27.66343198700906</v>
       </c>
@@ -4736,9 +5177,18 @@
       <c r="J51" t="n">
         <v>0.4134</v>
       </c>
+      <c r="K51" t="n">
+        <v>0.4005492439271998</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.399725661903271</v>
+      </c>
       <c r="M51" t="n">
         <v>34.7217</v>
       </c>
+      <c r="N51" t="n">
+        <v>34.88888865237463</v>
+      </c>
       <c r="O51" t="n">
         <v>27.86199170274813</v>
       </c>
@@ -4822,9 +5272,18 @@
       <c r="J52" t="n">
         <v>0.8479</v>
       </c>
+      <c r="K52" t="n">
+        <v>0.8234014411517872</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.8237382476966327</v>
+      </c>
       <c r="M52" t="n">
         <v>34.8584</v>
       </c>
+      <c r="N52" t="n">
+        <v>35.02594699136187</v>
+      </c>
       <c r="O52" t="n">
         <v>27.94539604200054</v>
       </c>
@@ -4908,9 +5367,18 @@
       <c r="J53" t="n">
         <v>0.6372</v>
       </c>
+      <c r="K53" t="n">
+        <v>0.6089139492645129</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.6090247111743792</v>
+      </c>
       <c r="M53" t="n">
         <v>34.8622</v>
       </c>
+      <c r="N53" t="n">
+        <v>35.02958542710861</v>
+      </c>
       <c r="O53" t="n">
         <v>27.96197905979579</v>
       </c>
@@ -4994,9 +5462,18 @@
       <c r="J54" t="n">
         <v>0.3077</v>
       </c>
+      <c r="K54" t="n">
+        <v>0.2711898164074017</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.2709636603782534</v>
+      </c>
       <c r="M54" t="n">
         <v>34.8733</v>
       </c>
+      <c r="N54" t="n">
+        <v>35.04059810041132</v>
+      </c>
       <c r="O54" t="n">
         <v>27.99102752974773</v>
       </c>
@@ -5080,9 +5557,18 @@
       <c r="J55" t="n">
         <v>0.0545</v>
       </c>
+      <c r="K55" t="n">
+        <v>0.009395540369354711</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.008906025149602193</v>
+      </c>
       <c r="M55" t="n">
         <v>34.8832</v>
       </c>
+      <c r="N55" t="n">
+        <v>35.05053938757884</v>
+      </c>
       <c r="O55" t="n">
         <v>28.01358058609594</v>
       </c>
@@ -5166,9 +5652,18 @@
       <c r="J56" t="n">
         <v>-0.2902</v>
       </c>
+      <c r="K56" t="n">
+        <v>-0.3603170664283632</v>
+      </c>
+      <c r="L56" t="n">
+        <v>-0.3611325943818454</v>
+      </c>
       <c r="M56" t="n">
         <v>34.912</v>
       </c>
+      <c r="N56" t="n">
+        <v>35.08008090966194</v>
+      </c>
       <c r="O56" t="n">
         <v>28.05634215745158</v>
       </c>
@@ -5252,9 +5747,18 @@
       <c r="J57" t="n">
         <v>-0.4002</v>
       </c>
+      <c r="K57" t="n">
+        <v>-0.5013043958548534</v>
+      </c>
+      <c r="L57" t="n">
+        <v>-0.5021816224500646</v>
+      </c>
       <c r="M57" t="n">
         <v>34.9422</v>
       </c>
+      <c r="N57" t="n">
+        <v>35.11096354813818</v>
+      </c>
       <c r="O57" t="n">
         <v>28.08804081586709</v>
       </c>
@@ -5338,9 +5842,18 @@
       <c r="J58" t="n">
         <v>-0.2562</v>
       </c>
+      <c r="K58" t="n">
+        <v>-0.5051171683796951</v>
+      </c>
+      <c r="L58" t="n">
+        <v>-0.5059364960282191</v>
+      </c>
       <c r="M58" t="n">
         <v>34.9591</v>
       </c>
+      <c r="N58" t="n">
+        <v>35.12830438256481</v>
+      </c>
       <c r="O58" t="n">
         <v>28.10212833992841</v>
       </c>
@@ -5424,9 +5937,18 @@
       <c r="J59" t="n">
         <v>-1.3927</v>
       </c>
+      <c r="K59" t="n">
+        <v>-1.380006175630191</v>
+      </c>
+      <c r="L59" t="n">
+        <v>-1.392721498935322</v>
+      </c>
       <c r="M59" t="n">
         <v>25.8748</v>
       </c>
+      <c r="N59" t="n">
+        <v>25.99916483947493</v>
+      </c>
       <c r="O59" t="n">
         <v>20.77330141109644</v>
       </c>
@@ -5510,9 +6032,18 @@
       <c r="J60" t="n">
         <v>0.3295</v>
       </c>
+      <c r="K60" t="n">
+        <v>0.3442607905523365</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.327578129842247</v>
+      </c>
       <c r="M60" t="n">
         <v>31.1531</v>
       </c>
+      <c r="N60" t="n">
+        <v>31.30353958987824</v>
+      </c>
       <c r="O60" t="n">
         <v>24.99139902403454</v>
       </c>
@@ -5596,9 +6127,18 @@
       <c r="J61" t="n">
         <v>-0.5846</v>
       </c>
+      <c r="K61" t="n">
+        <v>-0.576137702398655</v>
+      </c>
+      <c r="L61" t="n">
+        <v>-0.5867732002306344</v>
+      </c>
       <c r="M61" t="n">
         <v>31.8773</v>
       </c>
+      <c r="N61" t="n">
+        <v>32.03163918488962</v>
+      </c>
       <c r="O61" t="n">
         <v>25.61728853410682</v>
       </c>
@@ -5682,9 +6222,18 @@
       <c r="J62" t="n">
         <v>-1.4689</v>
       </c>
+      <c r="K62" t="n">
+        <v>-1.467402968524079</v>
+      </c>
+      <c r="L62" t="n">
+        <v>-1.473051171800113</v>
+      </c>
       <c r="M62" t="n">
         <v>33.1184</v>
       </c>
+      <c r="N62" t="n">
+        <v>33.27912138066601</v>
+      </c>
       <c r="O62" t="n">
         <v>26.65001785796289</v>
       </c>
@@ -5768,9 +6317,18 @@
       <c r="J63" t="n">
         <v>-0.3448</v>
       </c>
+      <c r="K63" t="n">
+        <v>-0.351598804002993</v>
+      </c>
+      <c r="L63" t="n">
+        <v>-0.3542269402544961</v>
+      </c>
       <c r="M63" t="n">
         <v>34.4319</v>
       </c>
+      <c r="N63" t="n">
+        <v>34.59801562437259</v>
+      </c>
       <c r="O63" t="n">
         <v>27.6680301102781</v>
       </c>
@@ -5854,9 +6412,18 @@
       <c r="J64" t="n">
         <v>0.422</v>
       </c>
+      <c r="K64" t="n">
+        <v>0.4084179780055459</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.4075994206128587</v>
+      </c>
       <c r="M64" t="n">
         <v>34.721</v>
       </c>
+      <c r="N64" t="n">
+        <v>34.88840067293821</v>
+      </c>
       <c r="O64" t="n">
         <v>27.86106449209478</v>
       </c>
@@ -5940,9 +6507,18 @@
       <c r="J65" t="n">
         <v>0.823</v>
       </c>
+      <c r="K65" t="n">
+        <v>0.7993926113031292</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.7996269495785445</v>
+      </c>
       <c r="M65" t="n">
         <v>34.8448</v>
       </c>
+      <c r="N65" t="n">
+        <v>35.01239713608638</v>
+      </c>
       <c r="O65" t="n">
         <v>27.93628200631042</v>
       </c>
@@ -6026,9 +6602,18 @@
       <c r="J66" t="n">
         <v>0.6296</v>
       </c>
+      <c r="K66" t="n">
+        <v>0.6014697080578906</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.6015552501874314</v>
+      </c>
       <c r="M66" t="n">
         <v>34.859</v>
       </c>
+      <c r="N66" t="n">
+        <v>35.02641260625971</v>
+      </c>
       <c r="O66" t="n">
         <v>27.95994709043634</v>
       </c>
@@ -6112,9 +6697,18 @@
       <c r="J67" t="n">
         <v>0.2837</v>
       </c>
+      <c r="K67" t="n">
+        <v>0.2474822007909063</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.2472180121815503</v>
+      </c>
       <c r="M67" t="n">
         <v>34.8711</v>
       </c>
+      <c r="N67" t="n">
+        <v>35.03842610296688</v>
+      </c>
       <c r="O67" t="n">
         <v>27.99060195404854</v>
       </c>
@@ -6198,9 +6792,18 @@
       <c r="J68" t="n">
         <v>0.0208</v>
       </c>
+      <c r="K68" t="n">
+        <v>-0.02389950220951684</v>
+      </c>
+      <c r="L68" t="n">
+        <v>-0.02444049086731005</v>
+      </c>
       <c r="M68" t="n">
         <v>34.8804</v>
       </c>
+      <c r="N68" t="n">
+        <v>35.04777877984304</v>
+      </c>
       <c r="O68" t="n">
         <v>28.01334653920571</v>
       </c>
@@ -6284,9 +6887,18 @@
       <c r="J69" t="n">
         <v>-0.2843</v>
       </c>
+      <c r="K69" t="n">
+        <v>-0.3544585734861402</v>
+      </c>
+      <c r="L69" t="n">
+        <v>-0.3552580886929553</v>
+      </c>
       <c r="M69" t="n">
         <v>34.9142</v>
       </c>
+      <c r="N69" t="n">
+        <v>35.08237496939837</v>
+      </c>
       <c r="O69" t="n">
         <v>28.05781838280222</v>
       </c>
@@ -6370,9 +6982,18 @@
       <c r="J70" t="n">
         <v>-0.4036</v>
       </c>
+      <c r="K70" t="n">
+        <v>-0.5045521333415</v>
+      </c>
+      <c r="L70" t="n">
+        <v>-0.5054297670363301</v>
+      </c>
       <c r="M70" t="n">
         <v>34.9432</v>
       </c>
+      <c r="N70" t="n">
+        <v>35.11199652489609</v>
+      </c>
       <c r="O70" t="n">
         <v>28.08894272575412</v>
       </c>
@@ -6456,9 +7077,18 @@
       <c r="J71" t="n">
         <v>-0.2655</v>
       </c>
+      <c r="K71" t="n">
+        <v>-0.5052191711455837</v>
+      </c>
+      <c r="L71" t="n">
+        <v>-0.5060389299260739</v>
+      </c>
       <c r="M71" t="n">
         <v>34.9589</v>
       </c>
+      <c r="N71" t="n">
+        <v>35.12822201168271</v>
+      </c>
       <c r="O71" t="n">
         <v>28.10198376329231</v>
       </c>
@@ -6542,9 +7172,18 @@
       <c r="J72" t="n">
         <v>-1.3592</v>
       </c>
+      <c r="K72" t="n">
+        <v>-1.346169873260266</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-1.359229857398885</v>
+      </c>
       <c r="M72" t="n">
         <v>26.3704</v>
       </c>
+      <c r="N72" t="n">
+        <v>26.49719026444345</v>
+      </c>
       <c r="O72" t="n">
         <v>21.17427355672339</v>
       </c>
@@ -6628,9 +7267,18 @@
       <c r="J73" t="n">
         <v>0.3873</v>
       </c>
+      <c r="K73" t="n">
+        <v>0.4049097245121457</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.3858446333957644</v>
+      </c>
       <c r="M73" t="n">
         <v>30.6287</v>
       </c>
+      <c r="N73" t="n">
+        <v>30.77647899525462</v>
+      </c>
       <c r="O73" t="n">
         <v>24.57314037784272</v>
       </c>
@@ -6714,9 +7362,18 @@
       <c r="J74" t="n">
         <v>-0.6534</v>
       </c>
+      <c r="K74" t="n">
+        <v>-0.644773788943432</v>
+      </c>
+      <c r="L74" t="n">
+        <v>-0.6552634990116775</v>
+      </c>
       <c r="M74" t="n">
         <v>31.8451</v>
       </c>
+      <c r="N74" t="n">
+        <v>31.99912544342783</v>
+      </c>
       <c r="O74" t="n">
         <v>25.5967655773145</v>
       </c>
@@ -6800,9 +7457,18 @@
       <c r="J75" t="n">
         <v>-1.4336</v>
       </c>
+      <c r="K75" t="n">
+        <v>-1.431894851885809</v>
+      </c>
+      <c r="L75" t="n">
+        <v>-1.437537190332451</v>
+      </c>
       <c r="M75" t="n">
         <v>33.1519</v>
       </c>
+      <c r="N75" t="n">
+        <v>33.31337517726308</v>
+      </c>
       <c r="O75" t="n">
         <v>26.67741280988298</v>
       </c>
@@ -6886,9 +7552,18 @@
       <c r="J76" t="n">
         <v>-0.3636</v>
       </c>
+      <c r="K76" t="n">
+        <v>-0.3698585162395948</v>
+      </c>
+      <c r="L76" t="n">
+        <v>-0.3725027974192069</v>
+      </c>
       <c r="M76" t="n">
         <v>34.43</v>
       </c>
+      <c r="N76" t="n">
+        <v>34.59615295842629</v>
+      </c>
       <c r="O76" t="n">
         <v>27.66807611214062</v>
       </c>
@@ -6972,9 +7647,18 @@
       <c r="J77" t="n">
         <v>0.377</v>
       </c>
+      <c r="K77" t="n">
+        <v>0.3643191819281815</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0.3634238771265536</v>
+      </c>
       <c r="M77" t="n">
         <v>34.714</v>
       </c>
+      <c r="N77" t="n">
+        <v>34.88117673522621</v>
+      </c>
       <c r="O77" t="n">
         <v>27.85799446511533</v>
       </c>
@@ -7034,9 +7718,18 @@
       <c r="J78" t="n">
         <v>0.8105</v>
       </c>
+      <c r="K78" t="n">
+        <v>0.7873251606209084</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0.7875889739859094</v>
+      </c>
       <c r="M78" t="n">
         <v>34.8526</v>
       </c>
+      <c r="N78" t="n">
+        <v>35.02018639104101</v>
+      </c>
       <c r="O78" t="n">
         <v>27.94329058733206</v>
       </c>
@@ -7120,9 +7813,18 @@
       <c r="J79" t="n">
         <v>0.5962</v>
       </c>
+      <c r="K79" t="n">
+        <v>0.568256032748041</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.5683100375387025</v>
+      </c>
       <c r="M79" t="n">
         <v>34.8603</v>
       </c>
+      <c r="N79" t="n">
+        <v>35.02766859610973</v>
+      </c>
       <c r="O79" t="n">
         <v>27.96305869186131</v>
       </c>
@@ -7206,9 +7908,18 @@
       <c r="J80" t="n">
         <v>0.2653</v>
       </c>
+      <c r="K80" t="n">
+        <v>0.229195448577803</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0.2289130334410632</v>
+      </c>
       <c r="M80" t="n">
         <v>34.8718</v>
       </c>
+      <c r="N80" t="n">
+        <v>35.03909348663387</v>
+      </c>
       <c r="O80" t="n">
         <v>27.99208641365044</v>
       </c>
@@ -7292,9 +8003,18 @@
       <c r="J81" t="n">
         <v>0.0107</v>
       </c>
+      <c r="K81" t="n">
+        <v>-0.03391797069428685</v>
+      </c>
+      <c r="L81" t="n">
+        <v>-0.03446319224958698</v>
+      </c>
       <c r="M81" t="n">
         <v>34.8822</v>
       </c>
+      <c r="N81" t="n">
+        <v>35.04954805605044</v>
+      </c>
       <c r="O81" t="n">
         <v>28.01508439962322</v>
       </c>
@@ -7378,9 +8098,18 @@
       <c r="J82" t="n">
         <v>-0.289</v>
       </c>
+      <c r="K82" t="n">
+        <v>-0.3570165654535475</v>
+      </c>
+      <c r="L82" t="n">
+        <v>-0.3578296174815858</v>
+      </c>
       <c r="M82" t="n">
         <v>34.9116</v>
       </c>
+      <c r="N82" t="n">
+        <v>35.07966681867813</v>
+      </c>
       <c r="O82" t="n">
         <v>28.05584878404306</v>
       </c>
@@ -7464,9 +8193,18 @@
       <c r="J83" t="n">
         <v>-0.4046</v>
       </c>
+      <c r="K83" t="n">
+        <v>-0.5055978462662115</v>
+      </c>
+      <c r="L83" t="n">
+        <v>-0.5064739218391369</v>
+      </c>
       <c r="M83" t="n">
         <v>34.944</v>
       </c>
+      <c r="N83" t="n">
+        <v>35.11279670790738</v>
+      </c>
       <c r="O83" t="n">
         <v>28.08963128538926</v>
       </c>
@@ -7550,9 +8288,18 @@
       <c r="J84" t="n">
         <v>-0.2628</v>
       </c>
+      <c r="K84" t="n">
+        <v>-0.5051247546574544</v>
+      </c>
+      <c r="L84" t="n">
+        <v>-0.5059441805582728</v>
+      </c>
       <c r="M84" t="n">
         <v>34.959</v>
       </c>
+      <c r="N84" t="n">
+        <v>35.12827998065082</v>
+      </c>
       <c r="O84" t="n">
         <v>28.10206633241955</v>
       </c>
@@ -7636,9 +8383,18 @@
       <c r="J85" t="n">
         <v>-1.3624</v>
       </c>
+      <c r="K85" t="n">
+        <v>-1.349305918450943</v>
+      </c>
+      <c r="L85" t="n">
+        <v>-1.362422322758593</v>
+      </c>
       <c r="M85" t="n">
         <v>25.7945</v>
       </c>
+      <c r="N85" t="n">
+        <v>25.91843364807759</v>
+      </c>
       <c r="O85" t="n">
         <v>20.70882886984123</v>
       </c>
@@ -7722,9 +8478,18 @@
       <c r="J86" t="n">
         <v>0.8756</v>
       </c>
+      <c r="K86" t="n">
+        <v>0.897107504366448</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0.8741444412079986</v>
+      </c>
       <c r="M86" t="n">
         <v>30.3419</v>
       </c>
+      <c r="N86" t="n">
+        <v>30.48816101334285</v>
+      </c>
       <c r="O86" t="n">
         <v>24.33251417947758</v>
       </c>
@@ -7808,9 +8573,18 @@
       <c r="J87" t="n">
         <v>-0.4644</v>
       </c>
+      <c r="K87" t="n">
+        <v>-0.4553056314198346</v>
+      </c>
+      <c r="L87" t="n">
+        <v>-0.4665780368270609</v>
+      </c>
       <c r="M87" t="n">
         <v>31.7998</v>
       </c>
+      <c r="N87" t="n">
+        <v>31.95375143546831</v>
+      </c>
       <c r="O87" t="n">
         <v>25.54839930501544</v>
       </c>
@@ -7894,9 +8668,18 @@
       <c r="J88" t="n">
         <v>-1.4235</v>
       </c>
+      <c r="K88" t="n">
+        <v>-1.422275463428188</v>
+      </c>
+      <c r="L88" t="n">
+        <v>-1.42790256659353</v>
+      </c>
       <c r="M88" t="n">
         <v>33.169</v>
       </c>
+      <c r="N88" t="n">
+        <v>33.3298794690602</v>
+      </c>
       <c r="O88" t="n">
         <v>26.69127257594278</v>
       </c>
@@ -7980,9 +8763,18 @@
       <c r="J89" t="n">
         <v>-0.365</v>
       </c>
+      <c r="K89" t="n">
+        <v>-0.3720038486049044</v>
+      </c>
+      <c r="L89" t="n">
+        <v>-0.3746692842949116</v>
+      </c>
       <c r="M89" t="n">
         <v>34.4246</v>
       </c>
+      <c r="N89" t="n">
+        <v>34.59071678386201</v>
+      </c>
       <c r="O89" t="n">
         <v>27.66543158217223</v>
       </c>
@@ -8066,9 +8858,18 @@
       <c r="J90" t="n">
         <v>0.375</v>
       </c>
+      <c r="K90" t="n">
+        <v>0.3614392196732974</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0.3605204193518582</v>
+      </c>
       <c r="M90" t="n">
         <v>34.7094</v>
       </c>
+      <c r="N90" t="n">
+        <v>34.87689305105568</v>
+      </c>
       <c r="O90" t="n">
         <v>27.8549861225199</v>
       </c>
@@ -8128,9 +8929,18 @@
       <c r="J91" t="n">
         <v>0.8199</v>
       </c>
+      <c r="K91" t="n">
+        <v>0.7955876896927174</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0.7958423882638057</v>
+      </c>
       <c r="M91" t="n">
         <v>34.8492</v>
       </c>
+      <c r="N91" t="n">
+        <v>35.0168477605953</v>
+      </c>
       <c r="O91" t="n">
         <v>27.9402531669798</v>
       </c>
@@ -8214,9 +9024,18 @@
       <c r="J92" t="n">
         <v>0.6428</v>
       </c>
+      <c r="K92" t="n">
+        <v>0.6145741668310286</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0.6146649290985026</v>
+      </c>
       <c r="M92" t="n">
         <v>34.8571</v>
       </c>
+      <c r="N92" t="n">
+        <v>35.02455334687016</v>
+      </c>
       <c r="O92" t="n">
         <v>27.95791334361297</v>
       </c>
@@ -8300,9 +9119,18 @@
       <c r="J93" t="n">
         <v>0.2675</v>
       </c>
+      <c r="K93" t="n">
+        <v>0.231395894541026</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.2310993852346128</v>
+      </c>
       <c r="M93" t="n">
         <v>34.8682</v>
       </c>
+      <c r="N93" t="n">
+        <v>35.0355485357936</v>
+      </c>
       <c r="O93" t="n">
         <v>27.98955830105319</v>
       </c>
@@ -8380,9 +9208,18 @@
       <c r="J94" t="n">
         <v>0.0176</v>
       </c>
+      <c r="K94" t="n">
+        <v>-0.02706040898542634</v>
+      </c>
+      <c r="L94" t="n">
+        <v>-0.02760887056722542</v>
+      </c>
       <c r="M94" t="n">
         <v>34.8795</v>
       </c>
+      <c r="N94" t="n">
+        <v>35.04691451784689</v>
+      </c>
       <c r="O94" t="n">
         <v>28.01287373957234</v>
       </c>
@@ -8466,9 +9303,18 @@
       <c r="J95" t="n">
         <v>-0.2919</v>
       </c>
+      <c r="K95" t="n">
+        <v>-0.361953913138944</v>
+      </c>
+      <c r="L95" t="n">
+        <v>-0.3627590518611183</v>
+      </c>
       <c r="M95" t="n">
         <v>34.9151</v>
       </c>
+      <c r="N95" t="n">
+        <v>35.0833235523716</v>
+      </c>
       <c r="O95" t="n">
         <v>28.05926695726043</v>
       </c>
@@ -8552,9 +9398,18 @@
       <c r="J96" t="n">
         <v>-0.4034</v>
       </c>
+      <c r="K96" t="n">
+        <v>-0.5043673032121686</v>
+      </c>
+      <c r="L96" t="n">
+        <v>-0.5052450486190629</v>
+      </c>
       <c r="M96" t="n">
         <v>34.9431</v>
       </c>
+      <c r="N96" t="n">
+        <v>35.11190039292207</v>
+      </c>
       <c r="O96" t="n">
         <v>28.08909685049593</v>
       </c>
@@ -8638,9 +9493,18 @@
       <c r="J97" t="n">
         <v>-0.2694</v>
       </c>
+      <c r="K97" t="n">
+        <v>-0.5050582747005929</v>
+      </c>
+      <c r="L97" t="n">
+        <v>-0.5058773677616286</v>
+      </c>
       <c r="M97" t="n">
         <v>34.959</v>
       </c>
+      <c r="N97" t="n">
+        <v>35.12834797936485</v>
+      </c>
       <c r="O97" t="n">
         <v>28.10244131400623</v>
       </c>
@@ -8724,9 +9588,18 @@
       <c r="J98" t="n">
         <v>-1.3398</v>
       </c>
+      <c r="K98" t="n">
+        <v>-1.326371098153732</v>
+      </c>
+      <c r="L98" t="n">
+        <v>-1.33981555536801</v>
+      </c>
       <c r="M98" t="n">
         <v>25.1384</v>
       </c>
+      <c r="N98" t="n">
+        <v>25.25913839668996</v>
+      </c>
       <c r="O98" t="n">
         <v>20.17680000230121</v>
       </c>
@@ -8810,9 +9683,18 @@
       <c r="J99" t="n">
         <v>0.6449</v>
       </c>
+      <c r="K99" t="n">
+        <v>0.6623158267189911</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0.6429396371697003</v>
+      </c>
       <c r="M99" t="n">
         <v>30.863</v>
       </c>
+      <c r="N99" t="n">
+        <v>31.01192702117911</v>
+      </c>
       <c r="O99" t="n">
         <v>24.74139673702575</v>
       </c>
@@ -8896,9 +9778,18 @@
       <c r="J100" t="n">
         <v>-0.5203</v>
       </c>
+      <c r="K100" t="n">
+        <v>-0.5118845983086661</v>
+      </c>
+      <c r="L100" t="n">
+        <v>-0.5228718004288964</v>
+      </c>
       <c r="M100" t="n">
         <v>31.8302</v>
       </c>
+      <c r="N100" t="n">
+        <v>31.98451795009831</v>
+      </c>
       <c r="O100" t="n">
         <v>25.57453985996403</v>
       </c>
@@ -8982,9 +9873,18 @@
       <c r="J101" t="n">
         <v>-1.4263</v>
       </c>
+      <c r="K101" t="n">
+        <v>-1.425129279510841</v>
+      </c>
+      <c r="L101" t="n">
+        <v>-1.430783848367797</v>
+      </c>
       <c r="M101" t="n">
         <v>33.1514</v>
       </c>
+      <c r="N101" t="n">
+        <v>33.31215973035504</v>
+      </c>
       <c r="O101" t="n">
         <v>26.67382041904034</v>
       </c>
@@ -9068,9 +9968,18 @@
       <c r="J102" t="n">
         <v>-0.2553</v>
       </c>
+      <c r="K102" t="n">
+        <v>-0.2630343207128421</v>
+      </c>
+      <c r="L102" t="n">
+        <v>-0.2655717584784094</v>
+      </c>
       <c r="M102" t="n">
         <v>34.4436</v>
       </c>
+      <c r="N102" t="n">
+        <v>34.6098635070766</v>
+      </c>
       <c r="O102" t="n">
         <v>27.67582537623343</v>
       </c>
@@ -9154,9 +10063,18 @@
       <c r="J103" t="n">
         <v>0.4168</v>
       </c>
+      <c r="K103" t="n">
+        <v>0.4026407883605051</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.4017907848949531</v>
+      </c>
       <c r="M103" t="n">
         <v>34.7155</v>
       </c>
+      <c r="N103" t="n">
+        <v>34.88311752819862</v>
+      </c>
       <c r="O103" t="n">
         <v>27.85764238474644</v>
       </c>
@@ -9240,9 +10158,18 @@
       <c r="J104" t="n">
         <v>0.7941</v>
       </c>
+      <c r="K104" t="n">
+        <v>0.7702717943100407</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0.770450850904093</v>
+      </c>
       <c r="M104" t="n">
         <v>34.8406</v>
       </c>
+      <c r="N104" t="n">
+        <v>35.00828152376996</v>
+      </c>
       <c r="O104" t="n">
         <v>27.93510649172208</v>
       </c>
@@ -9326,9 +10253,18 @@
       <c r="J105" t="n">
         <v>0.6448</v>
       </c>
+      <c r="K105" t="n">
+        <v>0.6165821799627658</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.6166717924064504</v>
+      </c>
       <c r="M105" t="n">
         <v>34.8564</v>
       </c>
+      <c r="N105" t="n">
+        <v>35.02389978168121</v>
+      </c>
       <c r="O105" t="n">
         <v>27.95714435577156</v>
       </c>
@@ -9412,9 +10348,18 @@
       <c r="J106" t="n">
         <v>0.2788</v>
       </c>
+      <c r="K106" t="n">
+        <v>0.2425876562925362</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0.2423043413900524</v>
+      </c>
       <c r="M106" t="n">
         <v>34.8682</v>
       </c>
+      <c r="N106" t="n">
+        <v>35.035584179428</v>
+      </c>
       <c r="O106" t="n">
         <v>27.98880247798684</v>
       </c>
@@ -9498,9 +10443,18 @@
       <c r="J107" t="n">
         <v>0.023</v>
       </c>
+      <c r="K107" t="n">
+        <v>-0.02169597317972004</v>
+      </c>
+      <c r="L107" t="n">
+        <v>-0.02223879586530387</v>
+      </c>
       <c r="M107" t="n">
         <v>34.8793</v>
       </c>
+      <c r="N107" t="n">
+        <v>35.04675215394757</v>
+      </c>
       <c r="O107" t="n">
         <v>28.0124761610823</v>
       </c>
@@ -9584,9 +10538,18 @@
       <c r="J108" t="n">
         <v>-0.2918</v>
       </c>
+      <c r="K108" t="n">
+        <v>-0.3618397335548224</v>
+      </c>
+      <c r="L108" t="n">
+        <v>-0.3626468768377721</v>
+      </c>
       <c r="M108" t="n">
         <v>34.9145</v>
       </c>
+      <c r="N108" t="n">
+        <v>35.08276271235992</v>
+      </c>
       <c r="O108" t="n">
         <v>28.05876524146856</v>
       </c>
@@ -9670,9 +10633,18 @@
       <c r="J109" t="n">
         <v>-0.4043</v>
       </c>
+      <c r="K109" t="n">
+        <v>-0.5052234520295383</v>
+      </c>
+      <c r="L109" t="n">
+        <v>-0.5061004598852004</v>
+      </c>
       <c r="M109" t="n">
         <v>34.9436</v>
       </c>
+      <c r="N109" t="n">
+        <v>35.11240664228162</v>
+      </c>
       <c r="O109" t="n">
         <v>28.089459156972</v>
       </c>
@@ -9756,9 +10728,18 @@
       <c r="J110" t="n">
         <v>-0.2756</v>
       </c>
+      <c r="K110" t="n">
+        <v>-0.5050806854713953</v>
+      </c>
+      <c r="L110" t="n">
+        <v>-0.5058998320719932</v>
+      </c>
       <c r="M110" t="n">
         <v>34.959</v>
       </c>
+      <c r="N110" t="n">
+        <v>35.12834125487422</v>
+      </c>
       <c r="O110" t="n">
         <v>28.10243696809584</v>
       </c>
@@ -9842,9 +10823,18 @@
       <c r="J111" t="n">
         <v>0.1557</v>
       </c>
+      <c r="K111" t="n">
+        <v>0.1887991811586351</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0.155624600301082</v>
+      </c>
       <c r="M111" t="n">
         <v>25.6193</v>
       </c>
+      <c r="N111" t="n">
+        <v>25.74237158053854</v>
+      </c>
       <c r="O111" t="n">
         <v>20.54140257835434</v>
       </c>
@@ -9928,9 +10918,18 @@
       <c r="J112" t="n">
         <v>0.1689</v>
       </c>
+      <c r="K112" t="n">
+        <v>0.2020760158986215</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0.1687303249755261</v>
+      </c>
       <c r="M112" t="n">
         <v>25.6194</v>
       </c>
+      <c r="N112" t="n">
+        <v>25.74234614602279</v>
+      </c>
       <c r="O112" t="n">
         <v>20.54079681078565</v>
       </c>
@@ -10014,9 +11013,18 @@
       <c r="J113" t="n">
         <v>-0.5445</v>
       </c>
+      <c r="K113" t="n">
+        <v>-0.5358550274085144</v>
+      </c>
+      <c r="L113" t="n">
+        <v>-0.546663266575084</v>
+      </c>
       <c r="M113" t="n">
         <v>31.8644</v>
       </c>
+      <c r="N113" t="n">
+        <v>32.01867467670142</v>
+      </c>
       <c r="O113" t="n">
         <v>25.60641843273856</v>
       </c>
@@ -10100,9 +11108,18 @@
       <c r="J114" t="n">
         <v>-1.3376</v>
       </c>
+      <c r="K114" t="n">
+        <v>-1.336084059866204</v>
+      </c>
+      <c r="L114" t="n">
+        <v>-1.341938910901555</v>
+      </c>
       <c r="M114" t="n">
         <v>33.1154</v>
       </c>
+      <c r="N114" t="n">
+        <v>33.27666374634168</v>
+      </c>
       <c r="O114" t="n">
         <v>26.64361101783311</v>
       </c>
@@ -10186,9 +11203,18 @@
       <c r="J115" t="n">
         <v>-0.1532</v>
       </c>
+      <c r="K115" t="n">
+        <v>-0.161074753716254</v>
+      </c>
+      <c r="L115" t="n">
+        <v>-0.1634563483026206</v>
+      </c>
       <c r="M115" t="n">
         <v>34.4686</v>
       </c>
+      <c r="N115" t="n">
+        <v>34.63529116818557</v>
+      </c>
       <c r="O115" t="n">
         <v>27.6858498468066</v>
       </c>
@@ -10272,9 +11298,18 @@
       <c r="J116" t="n">
         <v>0.4177</v>
       </c>
+      <c r="K116" t="n">
+        <v>0.4036492168934323</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0.4027817291568404</v>
+      </c>
       <c r="M116" t="n">
         <v>34.7116</v>
       </c>
+      <c r="N116" t="n">
+        <v>34.87937264553957</v>
+      </c>
       <c r="O116" t="n">
         <v>27.854380372479</v>
       </c>
@@ -10358,9 +11393,18 @@
       <c r="J117" t="n">
         <v>0.8361</v>
       </c>
+      <c r="K117" t="n">
+        <v>0.811504200274073</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0.8117594144449167</v>
+      </c>
       <c r="M117" t="n">
         <v>34.8458</v>
       </c>
+      <c r="N117" t="n">
+        <v>35.01370995962112</v>
+      </c>
       <c r="O117" t="n">
         <v>27.93624000050477</v>
       </c>
@@ -10444,9 +11488,18 @@
       <c r="J118" t="n">
         <v>0.7005</v>
       </c>
+      <c r="K118" t="n">
+        <v>0.671886363517629</v>
+      </c>
+      <c r="L118" t="n">
+        <v>0.6720480586213696</v>
+      </c>
       <c r="M118" t="n">
         <v>34.858</v>
       </c>
+      <c r="N118" t="n">
+        <v>35.02557297022535</v>
+      </c>
       <c r="O118" t="n">
         <v>27.95499001175358</v>
       </c>
@@ -10506,9 +11559,18 @@
       <c r="J119" t="n">
         <v>0.351</v>
       </c>
+      <c r="K119" t="n">
+        <v>0.3142119026063919</v>
+      </c>
+      <c r="L119" t="n">
+        <v>0.3140289060041298</v>
+      </c>
       <c r="M119" t="n">
         <v>34.8716</v>
       </c>
+      <c r="N119" t="n">
+        <v>35.0391024532609</v>
+      </c>
       <c r="O119" t="n">
         <v>27.98723232115913</v>
       </c>
@@ -10592,9 +11654,18 @@
       <c r="J120" t="n">
         <v>0.1023</v>
       </c>
+      <c r="K120" t="n">
+        <v>0.05681568083555241</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0.05637268283375971</v>
+      </c>
       <c r="M120" t="n">
         <v>34.8808</v>
       </c>
+      <c r="N120" t="n">
+        <v>35.04833682067668</v>
+      </c>
       <c r="O120" t="n">
         <v>28.00923879765446</v>
       </c>
@@ -10678,9 +11749,18 @@
       <c r="J121" t="n">
         <v>-0.2747</v>
       </c>
+      <c r="K121" t="n">
+        <v>-0.344930590485541</v>
+      </c>
+      <c r="L121" t="n">
+        <v>-0.3457341666989533</v>
+      </c>
       <c r="M121" t="n">
         <v>34.91</v>
       </c>
+      <c r="N121" t="n">
+        <v>35.07826564091899</v>
+      </c>
       <c r="O121" t="n">
         <v>28.05395320587104</v>
       </c>
@@ -10764,9 +11844,18 @@
       <c r="J122" t="n">
         <v>-0.2624</v>
       </c>
+      <c r="K122" t="n">
+        <v>-0.5043359256759826</v>
+      </c>
+      <c r="L122" t="n">
+        <v>-0.5051527199736058</v>
+      </c>
       <c r="M122" t="n">
         <v>34.9592</v>
       </c>
+      <c r="N122" t="n">
+        <v>35.12872283656989</v>
+      </c>
       <c r="O122" t="n">
         <v>28.10230875162483</v>
       </c>
@@ -10850,9 +11939,18 @@
       <c r="J123" t="n">
         <v>-1.3859</v>
       </c>
+      <c r="K123" t="n">
+        <v>-1.373103352433639</v>
+      </c>
+      <c r="L123" t="n">
+        <v>-1.385917878921275</v>
+      </c>
       <c r="M123" t="n">
         <v>25.6407</v>
       </c>
+      <c r="N123" t="n">
+        <v>25.76382055853517</v>
+      </c>
       <c r="O123" t="n">
         <v>20.58257225646992</v>
       </c>
@@ -10912,9 +12010,18 @@
       <c r="J124" t="n">
         <v>0.5305</v>
       </c>
+      <c r="K124" t="n">
+        <v>0.5465975185060218</v>
+      </c>
+      <c r="L124" t="n">
+        <v>0.5283568485001908</v>
+      </c>
       <c r="M124" t="n">
         <v>30.998</v>
       </c>
+      <c r="N124" t="n">
+        <v>31.14776769779265</v>
+      </c>
       <c r="O124" t="n">
         <v>24.8576741393772</v>
       </c>
@@ -10998,9 +12105,18 @@
       <c r="J125" t="n">
         <v>-0.5247000000000001</v>
       </c>
+      <c r="K125" t="n">
+        <v>-0.5161078119097426</v>
+      </c>
+      <c r="L125" t="n">
+        <v>-0.5270597416542178</v>
+      </c>
       <c r="M125" t="n">
         <v>31.8375</v>
       </c>
+      <c r="N125" t="n">
+        <v>31.99179497895178</v>
+      </c>
       <c r="O125" t="n">
         <v>25.57091329219702</v>
       </c>
@@ -11084,9 +12200,18 @@
       <c r="J126" t="n">
         <v>-1.4289</v>
       </c>
+      <c r="K126" t="n">
+        <v>-1.427675112508666</v>
+      </c>
+      <c r="L126" t="n">
+        <v>-1.433389588724987</v>
+      </c>
       <c r="M126" t="n">
         <v>33.1157</v>
       </c>
+      <c r="N126" t="n">
+        <v>33.27627205714616</v>
+      </c>
       <c r="O126" t="n">
         <v>26.649561488171</v>
       </c>
@@ -11146,9 +12271,18 @@
       <c r="J127" t="n">
         <v>-0.2191</v>
       </c>
+      <c r="K127" t="n">
+        <v>-0.2270061676642789</v>
+      </c>
+      <c r="L127" t="n">
+        <v>-0.2294851917952438</v>
+      </c>
       <c r="M127" t="n">
         <v>34.4535</v>
       </c>
+      <c r="N127" t="n">
+        <v>34.61993763555971</v>
+      </c>
       <c r="O127" t="n">
         <v>27.68605887350395</v>
       </c>
@@ -11208,9 +12342,18 @@
       <c r="J128" t="n">
         <v>0.4455</v>
       </c>
+      <c r="K128" t="n">
+        <v>0.4310274748380453</v>
+      </c>
+      <c r="L128" t="n">
+        <v>0.4302499090324328</v>
+      </c>
       <c r="M128" t="n">
         <v>34.7246</v>
       </c>
+      <c r="N128" t="n">
+        <v>34.89236180461</v>
+      </c>
       <c r="O128" t="n">
         <v>27.86377114679908</v>
       </c>
@@ -11294,9 +12437,18 @@
       <c r="J129" t="n">
         <v>0.7637</v>
       </c>
+      <c r="K129" t="n">
+        <v>0.7415237875199607</v>
+      </c>
+      <c r="L129" t="n">
+        <v>0.7416375898689345</v>
+      </c>
       <c r="M129" t="n">
         <v>34.8344</v>
       </c>
+      <c r="N129" t="n">
+        <v>35.00219775056514</v>
+      </c>
       <c r="O129" t="n">
         <v>27.93152386522229</v>
       </c>
@@ -11380,9 +12532,18 @@
       <c r="J130" t="n">
         <v>0.6014</v>
       </c>
+      <c r="K130" t="n">
+        <v>0.5734442405025387</v>
+      </c>
+      <c r="L130" t="n">
+        <v>0.5734686053909078</v>
+      </c>
       <c r="M130" t="n">
         <v>34.8533</v>
       </c>
+      <c r="N130" t="n">
+        <v>35.02083193233205</v>
+      </c>
       <c r="O130" t="n">
         <v>27.95714629163626</v>
       </c>
@@ -11442,9 +12603,18 @@
       <c r="J131" t="n">
         <v>0.2771</v>
       </c>
+      <c r="K131" t="n">
+        <v>0.2409855401579424</v>
+      </c>
+      <c r="L131" t="n">
+        <v>0.2406957854556774</v>
+      </c>
       <c r="M131" t="n">
         <v>34.8672</v>
       </c>
+      <c r="N131" t="n">
+        <v>35.0346139385127</v>
+      </c>
       <c r="O131" t="n">
         <v>27.98780518071999</v>
       </c>
@@ -11528,9 +12698,18 @@
       <c r="J132" t="n">
         <v>0.0257</v>
       </c>
+      <c r="K132" t="n">
+        <v>-0.01892568304661469</v>
+      </c>
+      <c r="L132" t="n">
+        <v>-0.01946376806685127</v>
+      </c>
       <c r="M132" t="n">
         <v>34.8796</v>
       </c>
+      <c r="N132" t="n">
+        <v>35.04709011962885</v>
+      </c>
       <c r="O132" t="n">
         <v>28.01221118491412</v>
       </c>
@@ -11614,9 +12793,18 @@
       <c r="J133" t="n">
         <v>-0.293</v>
       </c>
+      <c r="K133" t="n">
+        <v>-0.3628834109760451</v>
+      </c>
+      <c r="L133" t="n">
+        <v>-0.3636901455997323</v>
+      </c>
       <c r="M133" t="n">
         <v>34.9149</v>
       </c>
+      <c r="N133" t="n">
+        <v>35.0832066127422</v>
+      </c>
       <c r="O133" t="n">
         <v>28.05889560468995</v>
       </c>
@@ -11676,9 +12864,18 @@
       <c r="J134" t="n">
         <v>-0.4036</v>
       </c>
+      <c r="K134" t="n">
+        <v>-0.5044441478377063</v>
+      </c>
+      <c r="L134" t="n">
+        <v>-0.505321239043921</v>
+      </c>
       <c r="M134" t="n">
         <v>34.9433</v>
       </c>
+      <c r="N134" t="n">
+        <v>35.11210830966436</v>
+      </c>
       <c r="O134" t="n">
         <v>28.08886346892064</v>
       </c>
@@ -11762,9 +12959,18 @@
       <c r="J135" t="n">
         <v>-0.3773</v>
       </c>
+      <c r="K135" t="n">
+        <v>-0.515576378545096</v>
+      </c>
+      <c r="L135" t="n">
+        <v>-0.5164239312862233</v>
+      </c>
       <c r="M135" t="n">
         <v>34.9553</v>
       </c>
+      <c r="N135" t="n">
+        <v>35.1242534439433</v>
+      </c>
       <c r="O135" t="n">
         <v>28.09920019924652</v>
       </c>
@@ -11848,9 +13054,18 @@
       <c r="J136" t="n">
         <v>-0.2881</v>
       </c>
+      <c r="K136" t="n">
+        <v>-0.5046899560591772</v>
+      </c>
+      <c r="L136" t="n">
+        <v>-0.5055078456091721</v>
+      </c>
       <c r="M136" t="n">
         <v>34.9592</v>
       </c>
+      <c r="N136" t="n">
+        <v>35.12854781176492</v>
+      </c>
       <c r="O136" t="n">
         <v>28.10218020287425</v>
       </c>
@@ -11910,9 +13125,18 @@
       <c r="J137" t="n">
         <v>-1.3463</v>
       </c>
+      <c r="K137" t="n">
+        <v>-1.332991902357316</v>
+      </c>
+      <c r="L137" t="n">
+        <v>-1.346310036392521</v>
+      </c>
       <c r="M137" t="n">
         <v>24.7561</v>
       </c>
+      <c r="N137" t="n">
+        <v>24.87498810834048</v>
+      </c>
       <c r="O137" t="n">
         <v>19.86619524344212</v>
       </c>
@@ -11996,9 +13220,18 @@
       <c r="J138" t="n">
         <v>0.2058</v>
       </c>
+      <c r="K138" t="n">
+        <v>0.2194769644022558</v>
+      </c>
+      <c r="L138" t="n">
+        <v>0.2037968749734058</v>
+      </c>
       <c r="M138" t="n">
         <v>31.2706</v>
       </c>
+      <c r="N138" t="n">
+        <v>31.42182383616493</v>
+      </c>
       <c r="O138" t="n">
         <v>25.09265830191885</v>
       </c>
@@ -12082,9 +13315,18 @@
       <c r="J139" t="n">
         <v>-0.5499000000000001</v>
       </c>
+      <c r="K139" t="n">
+        <v>-0.5414065154934139</v>
+      </c>
+      <c r="L139" t="n">
+        <v>-0.5521877508691765</v>
+      </c>
       <c r="M139" t="n">
         <v>31.867</v>
       </c>
+      <c r="N139" t="n">
+        <v>32.02156682533701</v>
+      </c>
       <c r="O139" t="n">
         <v>25.59669640511879</v>
       </c>
@@ -12168,9 +13410,18 @@
       <c r="J140" t="n">
         <v>-1.4211</v>
       </c>
+      <c r="K140" t="n">
+        <v>-1.420024771057457</v>
+      </c>
+      <c r="L140" t="n">
+        <v>-1.425669012712826</v>
+      </c>
       <c r="M140" t="n">
         <v>33.1614</v>
       </c>
+      <c r="N140" t="n">
+        <v>33.32216188285894</v>
+      </c>
       <c r="O140" t="n">
         <v>26.67655591260313</v>
       </c>
@@ -12254,9 +13505,18 @@
       <c r="J141" t="n">
         <v>-0.2268</v>
       </c>
+      <c r="K141" t="n">
+        <v>-0.2351777350864862</v>
+      </c>
+      <c r="L141" t="n">
+        <v>-0.2377059880567401</v>
+      </c>
       <c r="M141" t="n">
         <v>34.4421</v>
       </c>
+      <c r="N141" t="n">
+        <v>34.60845875946625</v>
+      </c>
       <c r="O141" t="n">
         <v>27.66994430071804</v>
       </c>
@@ -12340,9 +13600,18 @@
       <c r="J142" t="n">
         <v>0.4165</v>
       </c>
+      <c r="K142" t="n">
+        <v>0.4007203290334934</v>
+      </c>
+      <c r="L142" t="n">
+        <v>0.3998871996922255</v>
+      </c>
       <c r="M142" t="n">
         <v>34.7194</v>
       </c>
+      <c r="N142" t="n">
+        <v>34.88691451636374</v>
+      </c>
       <c r="O142" t="n">
         <v>27.86055606649575</v>
       </c>
@@ -12426,9 +13695,18 @@
       <c r="J143" t="n">
         <v>0.6168</v>
       </c>
+      <c r="K143" t="n">
+        <v>0.596142144892961</v>
+      </c>
+      <c r="L143" t="n">
+        <v>0.5960190955817672</v>
+      </c>
       <c r="M143" t="n">
         <v>34.82</v>
       </c>
+      <c r="N143" t="n">
+        <v>34.98774364334056</v>
+      </c>
       <c r="O143" t="n">
         <v>27.92907620221195</v>
       </c>
@@ -12512,9 +13790,18 @@
       <c r="J144" t="n">
         <v>0.3433</v>
       </c>
+      <c r="K144" t="n">
+        <v>0.3169246482579326</v>
+      </c>
+      <c r="L144" t="n">
+        <v>0.3166982493483874</v>
+      </c>
       <c r="M144" t="n">
         <v>34.8619</v>
       </c>
+      <c r="N144" t="n">
+        <v>35.02945659822967</v>
+      </c>
       <c r="O144" t="n">
         <v>27.97935555045137</v>
       </c>
@@ -12598,9 +13885,18 @@
       <c r="J145" t="n">
         <v>0.1098</v>
       </c>
+      <c r="K145" t="n">
+        <v>0.07494214733002275</v>
+      </c>
+      <c r="L145" t="n">
+        <v>0.07448928618608756</v>
+      </c>
       <c r="M145" t="n">
         <v>34.8739</v>
       </c>
+      <c r="N145" t="n">
+        <v>35.0413293785355</v>
+      </c>
       <c r="O145" t="n">
         <v>28.00264000128186</v>
       </c>
@@ -12684,9 +13980,18 @@
       <c r="J146" t="n">
         <v>-0.3236</v>
       </c>
+      <c r="K146" t="n">
+        <v>-0.3932184451497329</v>
+      </c>
+      <c r="L146" t="n">
+        <v>-0.3940551460038498</v>
+      </c>
       <c r="M146" t="n">
         <v>34.9169</v>
       </c>
+      <c r="N146" t="n">
+        <v>35.08519493276584</v>
+      </c>
       <c r="O146" t="n">
         <v>28.06194377956876</v>
       </c>
@@ -12770,9 +14075,18 @@
       <c r="J147" t="n">
         <v>-0.4046</v>
       </c>
+      <c r="K147" t="n">
+        <v>-0.5055114756972775</v>
+      </c>
+      <c r="L147" t="n">
+        <v>-0.506385830695895</v>
+      </c>
       <c r="M147" t="n">
         <v>34.9445</v>
       </c>
+      <c r="N147" t="n">
+        <v>35.11324182364706</v>
+      </c>
       <c r="O147" t="n">
         <v>28.08986623809142</v>
       </c>
@@ -12856,9 +14170,18 @@
       <c r="J148" t="n">
         <v>-0.3048</v>
       </c>
+      <c r="K148" t="n">
+        <v>-0.5032721107596825</v>
+      </c>
+      <c r="L148" t="n">
+        <v>-0.5040890724754045</v>
+      </c>
       <c r="M148" t="n">
         <v>34.959</v>
       </c>
+      <c r="N148" t="n">
+        <v>35.12829422743192</v>
+      </c>
       <c r="O148" t="n">
         <v>28.1017829102957</v>
       </c>
@@ -12942,9 +14265,18 @@
       <c r="J149" t="n">
         <v>-0.5917</v>
       </c>
+      <c r="K149" t="n">
+        <v>-0.5815205166120332</v>
+      </c>
+      <c r="L149" t="n">
+        <v>-0.5931499670148441</v>
+      </c>
       <c r="M149" t="n">
         <v>31.506</v>
       </c>
+      <c r="N149" t="n">
+        <v>31.65848380279505</v>
+      </c>
       <c r="O149" t="n">
         <v>25.31492573212563</v>
       </c>
@@ -13028,9 +14360,18 @@
       <c r="J150" t="n">
         <v>-0.899</v>
       </c>
+      <c r="K150" t="n">
+        <v>-0.8911381456474692</v>
+      </c>
+      <c r="L150" t="n">
+        <v>-0.90061802244551</v>
+      </c>
       <c r="M150" t="n">
         <v>31.9147</v>
       </c>
+      <c r="N150" t="n">
+        <v>32.06963936751327</v>
+      </c>
       <c r="O150" t="n">
         <v>25.65139325633209</v>
       </c>
@@ -13114,9 +14455,18 @@
       <c r="J151" t="n">
         <v>-1.2913</v>
       </c>
+      <c r="K151" t="n">
+        <v>-1.289266589050883</v>
+      </c>
+      <c r="L151" t="n">
+        <v>-1.295057839528229</v>
+      </c>
       <c r="M151" t="n">
         <v>33.1826</v>
       </c>
+      <c r="N151" t="n">
+        <v>33.34472379952997</v>
+      </c>
       <c r="O151" t="n">
         <v>26.69908029087446</v>
       </c>
@@ -13200,9 +14550,18 @@
       <c r="J152" t="n">
         <v>-0.2297</v>
       </c>
+      <c r="K152" t="n">
+        <v>-0.2357079695537902</v>
+      </c>
+      <c r="L152" t="n">
+        <v>-0.238304318732191</v>
+      </c>
       <c r="M152" t="n">
         <v>34.4245</v>
       </c>
+      <c r="N152" t="n">
+        <v>34.59106360344268</v>
+      </c>
       <c r="O152" t="n">
         <v>27.65837560145974</v>
       </c>
@@ -13286,9 +14645,18 @@
       <c r="J153" t="n">
         <v>0.4187</v>
       </c>
+      <c r="K153" t="n">
+        <v>0.4063193856838993</v>
+      </c>
+      <c r="L153" t="n">
+        <v>0.4054513381086807</v>
+      </c>
       <c r="M153" t="n">
         <v>34.7111</v>
       </c>
+      <c r="N153" t="n">
+        <v>34.87875460194836</v>
+      </c>
       <c r="O153" t="n">
         <v>27.85344730936117</v>
       </c>
@@ -13372,9 +14740,18 @@
       <c r="J154" t="n">
         <v>0.731</v>
       </c>
+      <c r="K154" t="n">
+        <v>0.7092566879809911</v>
+      </c>
+      <c r="L154" t="n">
+        <v>0.7093180614338906</v>
+      </c>
       <c r="M154" t="n">
         <v>34.8314</v>
       </c>
+      <c r="N154" t="n">
+        <v>34.99910981853481</v>
+      </c>
       <c r="O154" t="n">
         <v>27.93116780403489</v>
       </c>
@@ -13458,9 +14835,18 @@
       <c r="J155" t="n">
         <v>0.5992</v>
       </c>
+      <c r="K155" t="n">
+        <v>0.5713015040565671</v>
+      </c>
+      <c r="L155" t="n">
+        <v>0.5713226516962323</v>
+      </c>
       <c r="M155" t="n">
         <v>34.8532</v>
       </c>
+      <c r="N155" t="n">
+        <v>35.02068227647169</v>
+      </c>
       <c r="O155" t="n">
         <v>27.95721147849326</v>
       </c>
@@ -13520,9 +14906,18 @@
       <c r="J156" t="n">
         <v>0.2986</v>
       </c>
+      <c r="K156" t="n">
+        <v>0.262267576899178</v>
+      </c>
+      <c r="L156" t="n">
+        <v>0.2620023199363238</v>
+      </c>
       <c r="M156" t="n">
         <v>34.8672</v>
       </c>
+      <c r="N156" t="n">
+        <v>35.03456325778269</v>
+      </c>
       <c r="O156" t="n">
         <v>27.98645315052454</v>
       </c>
@@ -13582,9 +14977,18 @@
       <c r="J157" t="n">
         <v>0.0679</v>
       </c>
+      <c r="K157" t="n">
+        <v>0.02281663310168143</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0.0223202092893008</v>
+      </c>
       <c r="M157" t="n">
         <v>34.8779</v>
       </c>
+      <c r="N157" t="n">
+        <v>35.04533915405328</v>
+      </c>
       <c r="O157" t="n">
         <v>28.00868020615985</v>
       </c>
@@ -13644,9 +15048,18 @@
       <c r="J158" t="n">
         <v>-0.2836</v>
       </c>
+      <c r="K158" t="n">
+        <v>-0.3536906386672301</v>
+      </c>
+      <c r="L158" t="n">
+        <v>-0.3544997734432437</v>
+      </c>
       <c r="M158" t="n">
         <v>34.9114</v>
       </c>
+      <c r="N158" t="n">
+        <v>35.07962124183612</v>
+      </c>
       <c r="O158" t="n">
         <v>28.05555479428631</v>
       </c>
@@ -13706,9 +15119,18 @@
       <c r="J159" t="n">
         <v>-0.3883</v>
       </c>
+      <c r="K159" t="n">
+        <v>-0.4947130927527485</v>
+      </c>
+      <c r="L159" t="n">
+        <v>-0.4955507355089064</v>
+      </c>
       <c r="M159" t="n">
         <v>34.9509</v>
       </c>
+      <c r="N159" t="n">
+        <v>35.11954119805186</v>
+      </c>
       <c r="O159" t="n">
         <v>28.0945448952059</v>
       </c>
@@ -13792,9 +15214,18 @@
       <c r="J160" t="n">
         <v>-1.0969</v>
       </c>
+      <c r="K160" t="n">
+        <v>-1.080147803002634</v>
+      </c>
+      <c r="L160" t="n">
+        <v>-1.096933751627253</v>
+      </c>
       <c r="M160" t="n">
         <v>25.3609</v>
       </c>
+      <c r="N160" t="n">
+        <v>25.48281189747834</v>
+      </c>
       <c r="O160" t="n">
         <v>20.36128417958548</v>
       </c>
@@ -13878,9 +15309,18 @@
       <c r="J161" t="n">
         <v>0.2279</v>
       </c>
+      <c r="K161" t="n">
+        <v>0.241493440560069</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0.2258732289124685</v>
+      </c>
       <c r="M161" t="n">
         <v>31.3103</v>
       </c>
+      <c r="N161" t="n">
+        <v>31.46155852992174</v>
+      </c>
       <c r="O161" t="n">
         <v>25.12341795135376</v>
       </c>
@@ -13964,9 +15404,18 @@
       <c r="J162" t="n">
         <v>-0.2461</v>
       </c>
+      <c r="K162" t="n">
+        <v>-0.2533582981487794</v>
+      </c>
+      <c r="L162" t="n">
+        <v>-0.2559541697570039</v>
+      </c>
       <c r="M162" t="n">
         <v>34.4269</v>
       </c>
+      <c r="N162" t="n">
+        <v>34.59345951748193</v>
+      </c>
       <c r="O162" t="n">
         <v>27.66091490226995</v>
       </c>
@@ -14050,9 +15499,18 @@
       <c r="J163" t="n">
         <v>0.4112</v>
       </c>
+      <c r="K163" t="n">
+        <v>0.3973814619636501</v>
+      </c>
+      <c r="L163" t="n">
+        <v>0.3965000821869682</v>
+      </c>
       <c r="M163" t="n">
         <v>34.71</v>
       </c>
+      <c r="N163" t="n">
+        <v>34.87773096686454</v>
+      </c>
       <c r="O163" t="n">
         <v>27.85356676536799</v>
       </c>
@@ -14136,9 +15594,18 @@
       <c r="J164" t="n">
         <v>0.7709</v>
       </c>
+      <c r="K164" t="n">
+        <v>0.7481927135648527</v>
+      </c>
+      <c r="L164" t="n">
+        <v>0.748303296993858</v>
+      </c>
       <c r="M164" t="n">
         <v>34.8324</v>
       </c>
+      <c r="N164" t="n">
+        <v>35.00025561788554</v>
+      </c>
       <c r="O164" t="n">
         <v>27.92968228098198</v>
       </c>
@@ -14222,9 +15689,18 @@
       <c r="J165" t="n">
         <v>0.6784</v>
       </c>
+      <c r="K165" t="n">
+        <v>0.6499384965793988</v>
+      </c>
+      <c r="L165" t="n">
+        <v>0.6500618499676298</v>
+      </c>
       <c r="M165" t="n">
         <v>34.8555</v>
       </c>
+      <c r="N165" t="n">
+        <v>35.02308405391604</v>
+      </c>
       <c r="O165" t="n">
         <v>27.95418152318553</v>
       </c>
@@ -14308,9 +15784,18 @@
       <c r="J166" t="n">
         <v>0.3518</v>
       </c>
+      <c r="K166" t="n">
+        <v>0.3150166063778375</v>
+      </c>
+      <c r="L166" t="n">
+        <v>0.3148169698953308</v>
+      </c>
       <c r="M166" t="n">
         <v>34.868</v>
       </c>
+      <c r="N166" t="n">
+        <v>35.03545970662685</v>
+      </c>
       <c r="O166" t="n">
         <v>27.98445210546083</v>
       </c>
@@ -14394,9 +15879,18 @@
       <c r="J167" t="n">
         <v>0.091</v>
       </c>
+      <c r="K167" t="n">
+        <v>0.04572770147748562</v>
+      </c>
+      <c r="L167" t="n">
+        <v>0.04525674990582809</v>
+      </c>
       <c r="M167" t="n">
         <v>34.8775</v>
       </c>
+      <c r="N167" t="n">
+        <v>35.04498807805364</v>
+      </c>
       <c r="O167" t="n">
         <v>28.00726376951047</v>
       </c>
@@ -14480,9 +15974,18 @@
       <c r="J168" t="n">
         <v>-0.2663</v>
       </c>
+      <c r="K168" t="n">
+        <v>-0.3365660344496422</v>
+      </c>
+      <c r="L168" t="n">
+        <v>-0.3373660706281572</v>
+      </c>
       <c r="M168" t="n">
         <v>34.9083</v>
       </c>
+      <c r="N168" t="n">
+        <v>35.07652197297659</v>
+      </c>
       <c r="O168" t="n">
         <v>28.05225549744046</v>
       </c>
@@ -14566,9 +16069,18 @@
       <c r="J169" t="n">
         <v>-0.3944</v>
       </c>
+      <c r="K169" t="n">
+        <v>-0.4954194368935659</v>
+      </c>
+      <c r="L169" t="n">
+        <v>-0.4962964193501245</v>
+      </c>
       <c r="M169" t="n">
         <v>34.9402</v>
       </c>
+      <c r="N169" t="n">
+        <v>35.10896269548876</v>
+      </c>
       <c r="O169" t="n">
         <v>28.08614934587263</v>
       </c>
@@ -14652,9 +16164,18 @@
       <c r="J170" t="n">
         <v>-0.2558</v>
       </c>
+      <c r="K170" t="n">
+        <v>-0.5046942217067147</v>
+      </c>
+      <c r="L170" t="n">
+        <v>-0.505512379078305</v>
+      </c>
       <c r="M170" t="n">
         <v>34.959</v>
       </c>
+      <c r="N170" t="n">
+        <v>35.12847540811957</v>
+      </c>
       <c r="O170" t="n">
         <v>28.10228851598276</v>
       </c>
@@ -14738,9 +16259,18 @@
       <c r="J171" t="n">
         <v>-1.3633</v>
       </c>
+      <c r="K171" t="n">
+        <v>-1.350199706564258</v>
+      </c>
+      <c r="L171" t="n">
+        <v>-1.363319732063738</v>
+      </c>
       <c r="M171" t="n">
         <v>25.5449</v>
       </c>
+      <c r="N171" t="n">
+        <v>25.66782214796277</v>
+      </c>
       <c r="O171" t="n">
         <v>20.49893923717184</v>
       </c>
@@ -14824,9 +16354,18 @@
       <c r="J172" t="n">
         <v>0.3149</v>
       </c>
+      <c r="K172" t="n">
+        <v>0.3292916033128021</v>
+      </c>
+      <c r="L172" t="n">
+        <v>0.3129218487237904</v>
+      </c>
       <c r="M172" t="n">
         <v>31.2146</v>
       </c>
+      <c r="N172" t="n">
+        <v>31.36572366375314</v>
+      </c>
       <c r="O172" t="n">
         <v>25.03526693465415</v>
       </c>
@@ -14910,9 +16449,18 @@
       <c r="J173" t="n">
         <v>-0.5139</v>
       </c>
+      <c r="K173" t="n">
+        <v>-0.5050202663350359</v>
+      </c>
+      <c r="L173" t="n">
+        <v>-0.5160760585820575</v>
+      </c>
       <c r="M173" t="n">
         <v>31.8141</v>
       </c>
+      <c r="N173" t="n">
+        <v>31.96881101242844</v>
+      </c>
       <c r="O173" t="n">
         <v>25.55529184442275</v>
       </c>
@@ -14996,9 +16544,18 @@
       <c r="J174" t="n">
         <v>-1.4902</v>
       </c>
+      <c r="K174" t="n">
+        <v>-1.48870972038365</v>
+      </c>
+      <c r="L174" t="n">
+        <v>-1.494267571147454</v>
+      </c>
       <c r="M174" t="n">
         <v>33.1514</v>
       </c>
+      <c r="N174" t="n">
+        <v>33.313288074285</v>
+      </c>
       <c r="O174" t="n">
         <v>26.67870988910568</v>
       </c>
@@ -15082,9 +16639,18 @@
       <c r="J175" t="n">
         <v>-0.2313</v>
       </c>
+      <c r="K175" t="n">
+        <v>-0.2385304172525523</v>
+      </c>
+      <c r="L175" t="n">
+        <v>-0.241040184645273</v>
+      </c>
       <c r="M175" t="n">
         <v>34.447</v>
       </c>
+      <c r="N175" t="n">
+        <v>34.61365334624634</v>
+      </c>
       <c r="O175" t="n">
         <v>27.67583134384472</v>
       </c>
@@ -15168,9 +16734,18 @@
       <c r="J176" t="n">
         <v>0.4111</v>
       </c>
+      <c r="K176" t="n">
+        <v>0.3977261682164838</v>
+      </c>
+      <c r="L176" t="n">
+        <v>0.3968569584188182</v>
+      </c>
       <c r="M176" t="n">
         <v>34.7125</v>
       </c>
+      <c r="N176" t="n">
+        <v>34.88014372976938</v>
+      </c>
       <c r="O176" t="n">
         <v>27.85524505060721</v>
       </c>
@@ -15254,9 +16829,18 @@
       <c r="J177" t="n">
         <v>0.7786999999999999</v>
       </c>
+      <c r="K177" t="n">
+        <v>0.7567277359963889</v>
+      </c>
+      <c r="L177" t="n">
+        <v>0.7568729698185078</v>
+      </c>
       <c r="M177" t="n">
         <v>34.837</v>
       </c>
+      <c r="N177" t="n">
+        <v>35.00486428561278</v>
+      </c>
       <c r="O177" t="n">
         <v>27.93292422672471</v>
       </c>
@@ -15340,9 +16924,18 @@
       <c r="J178" t="n">
         <v>0.5909</v>
       </c>
+      <c r="K178" t="n">
+        <v>0.5629538787783199</v>
+      </c>
+      <c r="L178" t="n">
+        <v>0.5629894286943039</v>
+      </c>
       <c r="M178" t="n">
         <v>34.8577</v>
       </c>
+      <c r="N178" t="n">
+        <v>35.02528670819557</v>
+      </c>
       <c r="O178" t="n">
         <v>27.96141020191726</v>
       </c>
@@ -15426,9 +17019,18 @@
       <c r="J179" t="n">
         <v>0.2486</v>
       </c>
+      <c r="K179" t="n">
+        <v>0.2125767378275818</v>
+      </c>
+      <c r="L179" t="n">
+        <v>0.2122686868268897</v>
+      </c>
       <c r="M179" t="n">
         <v>34.8703</v>
       </c>
+      <c r="N179" t="n">
+        <v>35.03776624883816</v>
+      </c>
       <c r="O179" t="n">
         <v>27.99208808139292</v>
       </c>
@@ -15512,9 +17114,18 @@
       <c r="J180" t="n">
         <v>0.0063</v>
       </c>
+      <c r="K180" t="n">
+        <v>-0.03830516923284729</v>
+      </c>
+      <c r="L180" t="n">
+        <v>-0.03885756152942752</v>
+      </c>
       <c r="M180" t="n">
         <v>34.8816</v>
       </c>
+      <c r="N180" t="n">
+        <v>35.04909078328691</v>
+      </c>
       <c r="O180" t="n">
         <v>28.01507632338394</v>
       </c>
@@ -15598,9 +17209,18 @@
       <c r="J181" t="n">
         <v>-0.1999</v>
       </c>
+      <c r="K181" t="n">
+        <v>-0.2711509762981131</v>
+      </c>
+      <c r="L181" t="n">
+        <v>-0.2718932636040765</v>
+      </c>
       <c r="M181" t="n">
         <v>34.9027</v>
       </c>
+      <c r="N181" t="n">
+        <v>35.07085304456035</v>
+      </c>
       <c r="O181" t="n">
         <v>28.04446774717121</v>
       </c>
@@ -15684,9 +17304,18 @@
       <c r="J182" t="n">
         <v>-0.3717</v>
       </c>
+      <c r="K182" t="n">
+        <v>-0.4731925675852698</v>
+      </c>
+      <c r="L182" t="n">
+        <v>-0.4740708329088114</v>
+      </c>
       <c r="M182" t="n">
         <v>34.9322</v>
       </c>
+      <c r="N182" t="n">
+        <v>35.10088771254976</v>
+      </c>
       <c r="O182" t="n">
         <v>28.07859180446394</v>
       </c>
@@ -15770,9 +17399,18 @@
       <c r="J183" t="n">
         <v>-0.2532</v>
       </c>
+      <c r="K183" t="n">
+        <v>-0.5047041346652915</v>
+      </c>
+      <c r="L183" t="n">
+        <v>-0.5055228119310338</v>
+      </c>
       <c r="M183" t="n">
         <v>34.9589</v>
       </c>
+      <c r="N183" t="n">
+        <v>35.12833544367348</v>
+      </c>
       <c r="O183" t="n">
         <v>28.10217180642508</v>
       </c>
@@ -15856,9 +17494,18 @@
       <c r="J184" t="n">
         <v>-1.2456</v>
       </c>
+      <c r="K184" t="n">
+        <v>-1.231593703289036</v>
+      </c>
+      <c r="L184" t="n">
+        <v>-1.245651929607974</v>
+      </c>
       <c r="M184" t="n">
         <v>27.1105</v>
       </c>
+      <c r="N184" t="n">
+        <v>27.24089878610512</v>
+      </c>
       <c r="O184" t="n">
         <v>21.77336730545665</v>
       </c>
@@ -15942,9 +17589,18 @@
       <c r="J185" t="n">
         <v>0.2594</v>
       </c>
+      <c r="K185" t="n">
+        <v>0.2746295897932041</v>
+      </c>
+      <c r="L185" t="n">
+        <v>0.2578026807429364</v>
+      </c>
       <c r="M185" t="n">
         <v>31.0359</v>
       </c>
+      <c r="N185" t="n">
+        <v>31.18653201954612</v>
+      </c>
       <c r="O185" t="n">
         <v>24.89510516769565</v>
       </c>
@@ -16028,9 +17684,18 @@
       <c r="J186" t="n">
         <v>-0.668</v>
       </c>
+      <c r="K186" t="n">
+        <v>-0.6598583752520357</v>
+      </c>
+      <c r="L186" t="n">
+        <v>-0.6699997453987134</v>
+      </c>
       <c r="M186" t="n">
         <v>31.9551</v>
       </c>
+      <c r="N186" t="n">
+        <v>32.11126915423451</v>
+      </c>
       <c r="O186" t="n">
         <v>25.68134208658466</v>
       </c>
@@ -16114,9 +17779,18 @@
       <c r="J187" t="n">
         <v>-1.3542</v>
       </c>
+      <c r="K187" t="n">
+        <v>-1.352267893046979</v>
+      </c>
+      <c r="L187" t="n">
+        <v>-1.357977054227676</v>
+      </c>
       <c r="M187" t="n">
         <v>33.1783</v>
       </c>
+      <c r="N187" t="n">
+        <v>33.34045413851217</v>
+      </c>
       <c r="O187" t="n">
         <v>26.69474752165138</v>
       </c>
@@ -16200,9 +17874,18 @@
       <c r="J188" t="n">
         <v>-0.1954</v>
       </c>
+      <c r="K188" t="n">
+        <v>-0.2015240470795047</v>
+      </c>
+      <c r="L188" t="n">
+        <v>-0.2040544320994003</v>
+      </c>
       <c r="M188" t="n">
         <v>34.4369</v>
       </c>
+      <c r="N188" t="n">
+        <v>34.60345006742988</v>
+      </c>
       <c r="O188" t="n">
         <v>27.66624407878271</v>
       </c>
@@ -16286,9 +17969,18 @@
       <c r="J189" t="n">
         <v>0.3856</v>
       </c>
+      <c r="K189" t="n">
+        <v>0.3737651186223432</v>
+      </c>
+      <c r="L189" t="n">
+        <v>0.3728711247620188</v>
+      </c>
       <c r="M189" t="n">
         <v>34.7121</v>
       </c>
+      <c r="N189" t="n">
+        <v>34.87963799920642</v>
+      </c>
       <c r="O189" t="n">
         <v>27.85607498954801</v>
       </c>
@@ -16372,9 +18064,18 @@
       <c r="J190" t="n">
         <v>0.7195</v>
       </c>
+      <c r="K190" t="n">
+        <v>0.6991298616951255</v>
+      </c>
+      <c r="L190" t="n">
+        <v>0.6991915738694743</v>
+      </c>
       <c r="M190" t="n">
         <v>34.8335</v>
       </c>
+      <c r="N190" t="n">
+        <v>35.00124727626004</v>
+      </c>
       <c r="O190" t="n">
         <v>27.93397678774295</v>
       </c>
@@ -16458,9 +18159,18 @@
       <c r="J191" t="n">
         <v>0.4918</v>
       </c>
+      <c r="K191" t="n">
+        <v>0.4645427193138879</v>
+      </c>
+      <c r="L191" t="n">
+        <v>0.4644512980308369</v>
+      </c>
       <c r="M191" t="n">
         <v>34.855</v>
       </c>
+      <c r="N191" t="n">
+        <v>35.02246521895754</v>
+      </c>
       <c r="O191" t="n">
         <v>27.96533742671932</v>
       </c>
@@ -16544,9 +18254,18 @@
       <c r="J192" t="n">
         <v>0.2119</v>
       </c>
+      <c r="K192" t="n">
+        <v>0.1762487667449473</v>
+      </c>
+      <c r="L192" t="n">
+        <v>0.1758932027867088</v>
+      </c>
       <c r="M192" t="n">
         <v>34.8693</v>
       </c>
+      <c r="N192" t="n">
+        <v>35.03666244170854</v>
+      </c>
       <c r="O192" t="n">
         <v>27.99354429714776</v>
       </c>
@@ -16606,9 +18325,18 @@
       <c r="J193" t="n">
         <v>-0.0115</v>
       </c>
+      <c r="K193" t="n">
+        <v>-0.05588710733626417</v>
+      </c>
+      <c r="L193" t="n">
+        <v>-0.0564627892608495</v>
+      </c>
       <c r="M193" t="n">
         <v>34.8811</v>
       </c>
+      <c r="N193" t="n">
+        <v>35.04851821200872</v>
+      </c>
       <c r="O193" t="n">
         <v>28.01571584121461</v>
       </c>
@@ -16668,9 +18396,18 @@
       <c r="J194" t="n">
         <v>-0.3096</v>
       </c>
+      <c r="K194" t="n">
+        <v>-0.3794071664312011</v>
+      </c>
+      <c r="L194" t="n">
+        <v>-0.3802363494190613</v>
+      </c>
       <c r="M194" t="n">
         <v>34.9144</v>
       </c>
+      <c r="N194" t="n">
+        <v>35.08267183141417</v>
+      </c>
       <c r="O194" t="n">
         <v>28.05955693213036</v>
       </c>
@@ -16730,9 +18467,18 @@
       <c r="J195" t="n">
         <v>-0.3983</v>
       </c>
+      <c r="K195" t="n">
+        <v>-0.4993232017540562</v>
+      </c>
+      <c r="L195" t="n">
+        <v>-0.5001843412802095</v>
+      </c>
       <c r="M195" t="n">
         <v>34.9459</v>
       </c>
+      <c r="N195" t="n">
+        <v>35.11470226152542</v>
+      </c>
       <c r="O195" t="n">
         <v>28.09114861989474</v>
       </c>
@@ -16816,9 +18562,18 @@
       <c r="J196" t="n">
         <v>-0.3619</v>
       </c>
+      <c r="K196" t="n">
+        <v>-0.4991353851416062</v>
+      </c>
+      <c r="L196" t="n">
+        <v>-0.4999524897947629</v>
+      </c>
       <c r="M196" t="n">
         <v>34.9578</v>
       </c>
+      <c r="N196" t="n">
+        <v>35.12677095311399</v>
+      </c>
       <c r="O196" t="n">
         <v>28.10085070831815</v>
       </c>
@@ -16902,9 +18657,18 @@
       <c r="J197" t="n">
         <v>-1.3878</v>
       </c>
+      <c r="K197" t="n">
+        <v>-1.37505738930236</v>
+      </c>
+      <c r="L197" t="n">
+        <v>-1.387826938384502</v>
+      </c>
       <c r="M197" t="n">
         <v>25.9817</v>
       </c>
+      <c r="N197" t="n">
+        <v>26.1067376527853</v>
+      </c>
       <c r="O197" t="n">
         <v>20.86032727244401</v>
       </c>
@@ -16988,9 +18752,18 @@
       <c r="J198" t="n">
         <v>0.2078</v>
       </c>
+      <c r="K198" t="n">
+        <v>0.2213205246985741</v>
+      </c>
+      <c r="L198" t="n">
+        <v>0.2058817442982894</v>
+      </c>
       <c r="M198" t="n">
         <v>31.3353</v>
       </c>
+      <c r="N198" t="n">
+        <v>31.48681088591976</v>
+      </c>
       <c r="O198" t="n">
         <v>25.14986306712626</v>
       </c>
@@ -17074,9 +18847,18 @@
       <c r="J199" t="n">
         <v>-0.5580000000000001</v>
       </c>
+      <c r="K199" t="n">
+        <v>-0.549341595757914</v>
+      </c>
+      <c r="L199" t="n">
+        <v>-0.5601155871384044</v>
+      </c>
       <c r="M199" t="n">
         <v>31.86</v>
       </c>
+      <c r="N199" t="n">
+        <v>32.01454472978516</v>
+      </c>
       <c r="O199" t="n">
         <v>25.59124218356033</v>
       </c>
@@ -17160,9 +18942,18 @@
       <c r="J200" t="n">
         <v>-1.4812</v>
       </c>
+      <c r="K200" t="n">
+        <v>-1.479587752304909</v>
+      </c>
+      <c r="L200" t="n">
+        <v>-1.485197120794305</v>
+      </c>
       <c r="M200" t="n">
         <v>33.129</v>
       </c>
+      <c r="N200" t="n">
+        <v>33.29095274420408</v>
+      </c>
       <c r="O200" t="n">
         <v>26.6567170266394</v>
       </c>
@@ -17246,9 +19037,18 @@
       <c r="J201" t="n">
         <v>-0.3251</v>
       </c>
+      <c r="K201" t="n">
+        <v>-0.3320857824012736</v>
+      </c>
+      <c r="L201" t="n">
+        <v>-0.3346946603143365</v>
+      </c>
       <c r="M201" t="n">
         <v>34.4341</v>
       </c>
+      <c r="N201" t="n">
+        <v>34.60050842357764</v>
+      </c>
       <c r="O201" t="n">
         <v>27.66867019479059</v>
       </c>
@@ -17308,9 +19108,18 @@
       <c r="J202" t="n">
         <v>0.3942</v>
       </c>
+      <c r="K202" t="n">
+        <v>0.3805943706521864</v>
+      </c>
+      <c r="L202" t="n">
+        <v>0.3797109387044569</v>
+      </c>
       <c r="M202" t="n">
         <v>34.713</v>
       </c>
+      <c r="N202" t="n">
+        <v>34.88049869302106</v>
+      </c>
       <c r="O202" t="n">
         <v>27.85682193344542</v>
       </c>
@@ -17394,9 +19203,18 @@
       <c r="J203" t="n">
         <v>0.8288</v>
       </c>
+      <c r="K203" t="n">
+        <v>0.806669205888059</v>
+      </c>
+      <c r="L203" t="n">
+        <v>0.80687641643358</v>
+      </c>
       <c r="M203" t="n">
         <v>34.8383</v>
       </c>
+      <c r="N203" t="n">
+        <v>35.00603742130645</v>
+      </c>
       <c r="O203" t="n">
         <v>27.93056029413333</v>
       </c>
@@ -17480,9 +19298,18 @@
       <c r="J204" t="n">
         <v>0.7359</v>
       </c>
+      <c r="K204" t="n">
+        <v>0.7069820578802745</v>
+      </c>
+      <c r="L204" t="n">
+        <v>0.7072128322930485</v>
+      </c>
       <c r="M204" t="n">
         <v>34.8634</v>
       </c>
+      <c r="N204" t="n">
+        <v>35.03093058712999</v>
+      </c>
       <c r="O204" t="n">
         <v>27.95689735659312</v>
       </c>
@@ -17566,9 +19393,18 @@
       <c r="J205" t="n">
         <v>0.4043</v>
       </c>
+      <c r="K205" t="n">
+        <v>0.3670054882746467</v>
+      </c>
+      <c r="L205" t="n">
+        <v>0.3669038208443376</v>
+      </c>
       <c r="M205" t="n">
         <v>34.8757</v>
       </c>
+      <c r="N205" t="n">
+        <v>35.04310977889625</v>
+      </c>
       <c r="O205" t="n">
         <v>27.98736836648845</v>
       </c>
@@ -17628,9 +19464,18 @@
       <c r="J206" t="n">
         <v>0.08210000000000001</v>
       </c>
+      <c r="K206" t="n">
+        <v>0.03679047840986154</v>
+      </c>
+      <c r="L206" t="n">
+        <v>0.03632054536013434</v>
+      </c>
       <c r="M206" t="n">
         <v>34.8802</v>
       </c>
+      <c r="N206" t="n">
+        <v>35.047606388582</v>
+      </c>
       <c r="O206" t="n">
         <v>28.00975136198781</v>
       </c>
@@ -17714,9 +19559,18 @@
       <c r="J207" t="n">
         <v>-0.2748</v>
       </c>
+      <c r="K207" t="n">
+        <v>-0.3450382953931878</v>
+      </c>
+      <c r="L207" t="n">
+        <v>-0.3458471685307215</v>
+      </c>
       <c r="M207" t="n">
         <v>34.9088</v>
       </c>
+      <c r="N207" t="n">
+        <v>35.07692407552118</v>
+      </c>
       <c r="O207" t="n">
         <v>28.05307735003316</v>
       </c>
@@ -17800,9 +19654,18 @@
       <c r="J208" t="n">
         <v>-0.3974</v>
       </c>
+      <c r="K208" t="n">
+        <v>-0.4984888125586252</v>
+      </c>
+      <c r="L208" t="n">
+        <v>-0.4993656725902006</v>
+      </c>
       <c r="M208" t="n">
         <v>34.9413</v>
       </c>
+      <c r="N208" t="n">
+        <v>35.11007395145734</v>
+      </c>
       <c r="O208" t="n">
         <v>28.08722955890448</v>
       </c>
@@ -17886,9 +19749,18 @@
       <c r="J209" t="n">
         <v>-0.2551</v>
       </c>
+      <c r="K209" t="n">
+        <v>-0.5048762791103656</v>
+      </c>
+      <c r="L209" t="n">
+        <v>-0.5056951865819739</v>
+      </c>
       <c r="M209" t="n">
         <v>34.959</v>
       </c>
+      <c r="N209" t="n">
+        <v>35.12833378088541</v>
+      </c>
       <c r="O209" t="n">
         <v>28.10205966444937</v>
       </c>
@@ -17972,9 +19844,18 @@
       <c r="J210" t="n">
         <v>-1.4008</v>
       </c>
+      <c r="K210" t="n">
+        <v>-1.388268647420441</v>
+      </c>
+      <c r="L210" t="n">
+        <v>-1.40082990543998</v>
+      </c>
       <c r="M210" t="n">
         <v>26.3271</v>
       </c>
+      <c r="N210" t="n">
+        <v>26.45388228116363</v>
+      </c>
       <c r="O210" t="n">
         <v>21.14195093154967</v>
       </c>
@@ -18058,9 +19939,18 @@
       <c r="J211" t="n">
         <v>0.2213</v>
       </c>
+      <c r="K211" t="n">
+        <v>0.2351662845608913</v>
+      </c>
+      <c r="L211" t="n">
+        <v>0.2196523498872708</v>
+      </c>
       <c r="M211" t="n">
         <v>31.3308</v>
       </c>
+      <c r="N211" t="n">
+        <v>31.48223255349566</v>
+      </c>
       <c r="O211" t="n">
         <v>25.14019828162282</v>
       </c>
@@ -18144,9 +20034,18 @@
       <c r="J212" t="n">
         <v>-0.504</v>
       </c>
+      <c r="K212" t="n">
+        <v>-0.4948265694875572</v>
+      </c>
+      <c r="L212" t="n">
+        <v>-0.5058624235048851</v>
+      </c>
       <c r="M212" t="n">
         <v>31.8338</v>
       </c>
+      <c r="N212" t="n">
+        <v>31.98804186327729</v>
+      </c>
       <c r="O212" t="n">
         <v>25.58264733514079</v>
       </c>
@@ -18230,9 +20129,18 @@
       <c r="J213" t="n">
         <v>-1.5079</v>
       </c>
+      <c r="K213" t="n">
+        <v>-1.505755881391483</v>
+      </c>
+      <c r="L213" t="n">
+        <v>-1.511352430220538</v>
+      </c>
       <c r="M213" t="n">
         <v>33.111</v>
       </c>
+      <c r="N213" t="n">
+        <v>33.27454012648749</v>
+      </c>
       <c r="O213" t="n">
         <v>26.64649095911045</v>
       </c>
@@ -18316,9 +20224,18 @@
       <c r="J214" t="n">
         <v>0.9056</v>
       </c>
+      <c r="K214" t="n">
+        <v>0.882805962314077</v>
+      </c>
+      <c r="L214" t="n">
+        <v>0.8831558103047984</v>
+      </c>
       <c r="M214" t="n">
         <v>34.8486</v>
       </c>
+      <c r="N214" t="n">
+        <v>35.01628963659086</v>
+      </c>
       <c r="O214" t="n">
         <v>27.93397049889018</v>
       </c>
@@ -18402,9 +20319,18 @@
       <c r="J215" t="n">
         <v>0.6622</v>
       </c>
+      <c r="K215" t="n">
+        <v>0.6338512573874162</v>
+      </c>
+      <c r="L215" t="n">
+        <v>0.6339704554989153</v>
+      </c>
       <c r="M215" t="n">
         <v>34.8583</v>
       </c>
+      <c r="N215" t="n">
+        <v>35.02576296900401</v>
+      </c>
       <c r="O215" t="n">
         <v>27.95744155819011</v>
       </c>
@@ -18488,9 +20414,18 @@
       <c r="J216" t="n">
         <v>0.4161</v>
       </c>
+      <c r="K216" t="n">
+        <v>0.3786947920534541</v>
+      </c>
+      <c r="L216" t="n">
+        <v>0.3786318611069719</v>
+      </c>
       <c r="M216" t="n">
         <v>34.8808</v>
       </c>
+      <c r="N216" t="n">
+        <v>35.04819125661086</v>
+      </c>
       <c r="O216" t="n">
         <v>27.99095252351299</v>
       </c>
@@ -18574,9 +20509,18 @@
       <c r="J217" t="n">
         <v>0.1473</v>
       </c>
+      <c r="K217" t="n">
+        <v>0.1013879828353977</v>
+      </c>
+      <c r="L217" t="n">
+        <v>0.1010264270310758</v>
+      </c>
       <c r="M217" t="n">
         <v>34.8873</v>
       </c>
+      <c r="N217" t="n">
+        <v>35.05469244077138</v>
+      </c>
       <c r="O217" t="n">
         <v>28.01197768130874</v>
       </c>
@@ -18660,9 +20604,18 @@
       <c r="J218" t="n">
         <v>-0.2667</v>
       </c>
+      <c r="K218" t="n">
+        <v>-0.3370162577954854</v>
+      </c>
+      <c r="L218" t="n">
+        <v>-0.3378127768924193</v>
+      </c>
       <c r="M218" t="n">
         <v>34.9095</v>
       </c>
+      <c r="N218" t="n">
+        <v>35.07757566804787</v>
+      </c>
       <c r="O218" t="n">
         <v>28.05322718812135</v>
       </c>
@@ -18746,9 +20699,18 @@
       <c r="J219" t="n">
         <v>-0.3981</v>
       </c>
+      <c r="K219" t="n">
+        <v>-0.4990939874671924</v>
+      </c>
+      <c r="L219" t="n">
+        <v>-0.4999690646904084</v>
+      </c>
       <c r="M219" t="n">
         <v>34.942</v>
       </c>
+      <c r="N219" t="n">
+        <v>35.11077834590935</v>
+      </c>
       <c r="O219" t="n">
         <v>28.08774360104439</v>
       </c>
@@ -18832,9 +20794,18 @@
       <c r="J220" t="n">
         <v>-0.2558</v>
       </c>
+      <c r="K220" t="n">
+        <v>-0.5044260194129764</v>
+      </c>
+      <c r="L220" t="n">
+        <v>-0.5052446139153063</v>
+      </c>
       <c r="M220" t="n">
         <v>34.959</v>
       </c>
+      <c r="N220" t="n">
+        <v>35.12825830986944</v>
+      </c>
       <c r="O220" t="n">
         <v>28.10211004999655</v>
       </c>
@@ -18918,9 +20889,18 @@
       <c r="J221" t="n">
         <v>-0.7423</v>
       </c>
+      <c r="K221" t="n">
+        <v>-0.7470863308434449</v>
+      </c>
+      <c r="L221" t="n">
+        <v>-0.7499536182937336</v>
+      </c>
       <c r="M221" t="n">
         <v>34.4185</v>
       </c>
+      <c r="N221" t="n">
+        <v>34.58521166015909</v>
+      </c>
       <c r="O221" t="n">
         <v>27.67410274388203</v>
       </c>
@@ -19004,9 +20984,18 @@
       <c r="J222" t="n">
         <v>0.407</v>
       </c>
+      <c r="K222" t="n">
+        <v>0.3946017226035057</v>
+      </c>
+      <c r="L222" t="n">
+        <v>0.3937324283682246</v>
+      </c>
       <c r="M222" t="n">
         <v>34.7134</v>
       </c>
+      <c r="N222" t="n">
+        <v>34.88071951853153</v>
+      </c>
       <c r="O222" t="n">
         <v>27.85544235927227</v>
       </c>
@@ -19090,9 +21079,18 @@
       <c r="J223" t="n">
         <v>-1.4618</v>
       </c>
+      <c r="K223" t="n">
+        <v>-1.450137992621704</v>
+      </c>
+      <c r="L223" t="n">
+        <v>-1.461834483569258</v>
+      </c>
       <c r="M223" t="n">
         <v>27.0706</v>
       </c>
+      <c r="N223" t="n">
+        <v>27.20077306374004</v>
+      </c>
       <c r="O223" t="n">
         <v>21.74360649011032</v>
       </c>
@@ -19176,9 +21174,18 @@
       <c r="J224" t="n">
         <v>-1.1792</v>
       </c>
+      <c r="K224" t="n">
+        <v>-1.166501697595459</v>
+      </c>
+      <c r="L224" t="n">
+        <v>-1.17954531420513</v>
+      </c>
       <c r="M224" t="n">
         <v>28.9616</v>
       </c>
+      <c r="N224" t="n">
+        <v>29.10132531998699</v>
+      </c>
       <c r="O224" t="n">
         <v>23.24772800343101</v>
       </c>
@@ -19262,9 +21269,18 @@
       <c r="J225" t="n">
         <v>-0.6566</v>
       </c>
+      <c r="K225" t="n">
+        <v>-0.6481093033839752</v>
+      </c>
+      <c r="L225" t="n">
+        <v>-0.6585436542851527</v>
+      </c>
       <c r="M225" t="n">
         <v>31.8611</v>
       </c>
+      <c r="N225" t="n">
+        <v>32.01568964567154</v>
+      </c>
       <c r="O225" t="n">
         <v>25.60963565471025</v>
       </c>
@@ -19348,9 +21364,18 @@
       <c r="J226" t="n">
         <v>-1.4492</v>
       </c>
+      <c r="K226" t="n">
+        <v>-1.447212497577903</v>
+      </c>
+      <c r="L226" t="n">
+        <v>-1.452835921353143</v>
+      </c>
       <c r="M226" t="n">
         <v>33.1493</v>
       </c>
+      <c r="N226" t="n">
+        <v>33.31115722588419</v>
+      </c>
       <c r="O226" t="n">
         <v>26.67714470363694</v>
       </c>
@@ -19434,9 +21459,18 @@
       <c r="J227" t="n">
         <v>-0.4599</v>
       </c>
+      <c r="K227" t="n">
+        <v>-0.4654352275448443</v>
+      </c>
+      <c r="L227" t="n">
+        <v>-0.4681136202641926</v>
+      </c>
       <c r="M227" t="n">
         <v>34.4341</v>
       </c>
+      <c r="N227" t="n">
+        <v>34.60009213142518</v>
+      </c>
       <c r="O227" t="n">
         <v>27.67387795717127</v>
       </c>
@@ -19496,9 +21530,18 @@
       <c r="J228" t="n">
         <v>0.3967</v>
       </c>
+      <c r="K228" t="n">
+        <v>0.3843487701573605</v>
+      </c>
+      <c r="L228" t="n">
+        <v>0.3835056506191751</v>
+      </c>
       <c r="M228" t="n">
         <v>34.7211</v>
       </c>
+      <c r="N228" t="n">
+        <v>34.88802263260153</v>
+      </c>
       <c r="O228" t="n">
         <v>27.86231490123487</v>
       </c>
@@ -19582,9 +21625,18 @@
       <c r="J229" t="n">
         <v>0.8438</v>
       </c>
+      <c r="K229" t="n">
+        <v>0.8203249021147387</v>
+      </c>
+      <c r="L229" t="n">
+        <v>0.8206497912910368</v>
+      </c>
       <c r="M229" t="n">
         <v>34.857</v>
       </c>
+      <c r="N229" t="n">
+        <v>35.02443834194921</v>
+      </c>
       <c r="O229" t="n">
         <v>27.94435440791131</v>
       </c>
@@ -19668,9 +21720,18 @@
       <c r="J230" t="n">
         <v>0.5881</v>
       </c>
+      <c r="K230" t="n">
+        <v>0.5601687433590554</v>
+      </c>
+      <c r="L230" t="n">
+        <v>0.5602274900950124</v>
+      </c>
       <c r="M230" t="n">
         <v>34.8631</v>
       </c>
+      <c r="N230" t="n">
+        <v>35.03037258592593</v>
+      </c>
       <c r="O230" t="n">
         <v>27.96565780063884</v>
       </c>
@@ -19754,9 +21815,18 @@
       <c r="J231" t="n">
         <v>0.2444</v>
       </c>
+      <c r="K231" t="n">
+        <v>0.2084444278596415</v>
+      </c>
+      <c r="L231" t="n">
+        <v>0.2081383751131975</v>
+      </c>
       <c r="M231" t="n">
         <v>34.872</v>
       </c>
+      <c r="N231" t="n">
+        <v>35.03922785820193</v>
+      </c>
       <c r="O231" t="n">
         <v>27.99353273518341</v>
       </c>
@@ -19840,9 +21910,18 @@
       <c r="J232" t="n">
         <v>0.0159</v>
       </c>
+      <c r="K232" t="n">
+        <v>-0.02870761866226352</v>
+      </c>
+      <c r="L232" t="n">
+        <v>-0.02924122514577782</v>
+      </c>
       <c r="M232" t="n">
         <v>34.8835</v>
       </c>
+      <c r="N232" t="n">
+        <v>35.0508071918385</v>
+      </c>
       <c r="O232" t="n">
         <v>28.01598190937148</v>
       </c>
@@ -19926,9 +22005,18 @@
       <c r="J233" t="n">
         <v>-0.4041</v>
       </c>
+      <c r="K233" t="n">
+        <v>-0.5050420836439972</v>
+      </c>
+      <c r="L233" t="n">
+        <v>-0.5059183931294966</v>
+      </c>
       <c r="M233" t="n">
         <v>34.9438</v>
       </c>
+      <c r="N233" t="n">
+        <v>35.11253559065725</v>
+      </c>
       <c r="O233" t="n">
         <v>28.08939721946922</v>
       </c>
@@ -20012,9 +22100,18 @@
       <c r="J234" t="n">
         <v>-0.262</v>
       </c>
+      <c r="K234" t="n">
+        <v>-0.5051116511561708</v>
+      </c>
+      <c r="L234" t="n">
+        <v>-0.5059314660342328</v>
+      </c>
       <c r="M234" t="n">
         <v>34.959</v>
       </c>
+      <c r="N234" t="n">
+        <v>35.12816786321155</v>
+      </c>
       <c r="O234" t="n">
         <v>28.10197554005299</v>
       </c>
@@ -20098,9 +22195,18 @@
       <c r="J235" t="n">
         <v>0.4311</v>
       </c>
+      <c r="K235" t="n">
+        <v>0.469871674583149</v>
+      </c>
+      <c r="L235" t="n">
+        <v>0.4310101272378093</v>
+      </c>
       <c r="M235" t="n">
         <v>24.8759</v>
       </c>
+      <c r="N235" t="n">
+        <v>24.99531410596256</v>
+      </c>
       <c r="O235" t="n">
         <v>19.94893386714625</v>
       </c>
@@ -20184,9 +22290,18 @@
       <c r="J236" t="n">
         <v>0.4746</v>
       </c>
+      <c r="K236" t="n">
+        <v>0.4945278469367992</v>
+      </c>
+      <c r="L236" t="n">
+        <v>0.473323651271994</v>
+      </c>
       <c r="M236" t="n">
         <v>30.2167</v>
       </c>
+      <c r="N236" t="n">
+        <v>30.36200855556258</v>
+      </c>
       <c r="O236" t="n">
         <v>24.22229369079218</v>
       </c>
@@ -20270,9 +22385,18 @@
       <c r="J237" t="n">
         <v>0.2218</v>
       </c>
+      <c r="K237" t="n">
+        <v>0.2357697791072066</v>
+      </c>
+      <c r="L237" t="n">
+        <v>0.2199452051200891</v>
+      </c>
       <c r="M237" t="n">
         <v>31.2517</v>
       </c>
+      <c r="N237" t="n">
+        <v>31.40225328233601</v>
+      </c>
       <c r="O237" t="n">
         <v>25.07503392158242</v>
       </c>
@@ -20332,9 +22456,18 @@
       <c r="J238" t="n">
         <v>-0.3146</v>
       </c>
+      <c r="K238" t="n">
+        <v>-0.297874809185197</v>
+      </c>
+      <c r="L238" t="n">
+        <v>-0.3164881345293887</v>
+      </c>
       <c r="M238" t="n">
         <v>29.4583</v>
       </c>
+      <c r="N238" t="n">
+        <v>29.60065862848967</v>
+      </c>
       <c r="O238" t="n">
         <v>23.65220462362993</v>
       </c>
@@ -20418,9 +22551,18 @@
       <c r="J239" t="n">
         <v>-1.2253</v>
       </c>
+      <c r="K239" t="n">
+        <v>-1.22016624024913</v>
+      </c>
+      <c r="L239" t="n">
+        <v>-1.227761206552499</v>
+      </c>
       <c r="M239" t="n">
         <v>32.3341</v>
       </c>
+      <c r="N239" t="n">
+        <v>32.49220478448782</v>
+      </c>
       <c r="O239" t="n">
         <v>26.00807070712017</v>
       </c>
@@ -20504,9 +22646,18 @@
       <c r="J240" t="n">
         <v>-1.3464</v>
       </c>
+      <c r="K240" t="n">
+        <v>-1.342688958497639</v>
+      </c>
+      <c r="L240" t="n">
+        <v>-1.349453097641779</v>
+      </c>
       <c r="M240" t="n">
         <v>32.6171</v>
       </c>
+      <c r="N240" t="n">
+        <v>32.77676089044205</v>
+      </c>
       <c r="O240" t="n">
         <v>26.24108043643787</v>
       </c>
@@ -20590,9 +22741,18 @@
       <c r="J241" t="n">
         <v>-1.4302</v>
       </c>
+      <c r="K241" t="n">
+        <v>-1.427894058435953</v>
+      </c>
+      <c r="L241" t="n">
+        <v>-1.433921049742325</v>
+      </c>
       <c r="M241" t="n">
         <v>32.9366</v>
       </c>
+      <c r="N241" t="n">
+        <v>33.09731179684491</v>
+      </c>
       <c r="O241" t="n">
         <v>26.50497770363245</v>
       </c>
@@ -20676,9 +22836,18 @@
       <c r="J242" t="n">
         <v>-1.3997</v>
       </c>
+      <c r="K242" t="n">
+        <v>-1.398033981745375</v>
+      </c>
+      <c r="L242" t="n">
+        <v>-1.403811316904279</v>
+      </c>
       <c r="M242" t="n">
         <v>33.1058</v>
       </c>
+      <c r="N242" t="n">
+        <v>33.26683671394919</v>
+      </c>
       <c r="O242" t="n">
         <v>26.64080879828566</v>
       </c>
@@ -20762,9 +22931,18 @@
       <c r="J243" t="n">
         <v>-1.1367</v>
       </c>
+      <c r="K243" t="n">
+        <v>-1.137215786623852</v>
+      </c>
+      <c r="L243" t="n">
+        <v>-1.142158398885463</v>
+      </c>
       <c r="M243" t="n">
         <v>33.6471</v>
       </c>
+      <c r="N243" t="n">
+        <v>33.81033236114111</v>
+      </c>
       <c r="O243" t="n">
         <v>27.07232544928979</v>
       </c>
@@ -20848,9 +23026,18 @@
       <c r="J244" t="n">
         <v>-0.6755</v>
       </c>
+      <c r="K244" t="n">
+        <v>-0.6793825238548686</v>
+      </c>
+      <c r="L244" t="n">
+        <v>-0.6830534543616057</v>
+      </c>
       <c r="M244" t="n">
         <v>34.1582</v>
       </c>
+      <c r="N244" t="n">
+        <v>34.32356553209475</v>
+      </c>
       <c r="O244" t="n">
         <v>27.4607738960774</v>
       </c>
@@ -20934,9 +23121,18 @@
       <c r="J245" t="n">
         <v>-0.2421</v>
       </c>
+      <c r="K245" t="n">
+        <v>-0.2490480226120725</v>
+      </c>
+      <c r="L245" t="n">
+        <v>-0.2516372412886431</v>
+      </c>
       <c r="M245" t="n">
         <v>34.4281</v>
       </c>
+      <c r="N245" t="n">
+        <v>34.59461751907028</v>
+      </c>
       <c r="O245" t="n">
         <v>27.66178921291703</v>
       </c>
@@ -21020,9 +23216,18 @@
       <c r="J246" t="n">
         <v>0.4411</v>
       </c>
+      <c r="K246" t="n">
+        <v>0.4272736290222598</v>
+      </c>
+      <c r="L246" t="n">
+        <v>0.4264779590397049</v>
+      </c>
       <c r="M246" t="n">
         <v>34.7216</v>
       </c>
+      <c r="N246" t="n">
+        <v>34.88942909061965</v>
+      </c>
       <c r="O246" t="n">
         <v>27.86084707376131</v>
       </c>
@@ -21106,9 +23311,18 @@
       <c r="J247" t="n">
         <v>0.6398</v>
       </c>
+      <c r="K247" t="n">
+        <v>0.6223484826767016</v>
+      </c>
+      <c r="L247" t="n">
+        <v>0.6220934138465131</v>
+      </c>
       <c r="M247" t="n">
         <v>34.7894</v>
       </c>
+      <c r="N247" t="n">
+        <v>34.95726303722828</v>
+      </c>
       <c r="O247" t="n">
         <v>27.90315239288452</v>
       </c>
@@ -21192,9 +23406,18 @@
       <c r="J248" t="n">
         <v>0.7401</v>
       </c>
+      <c r="K248" t="n">
+        <v>0.7181929134718307</v>
+      </c>
+      <c r="L248" t="n">
+        <v>0.7182682469251257</v>
+      </c>
       <c r="M248" t="n">
         <v>34.832</v>
       </c>
+      <c r="N248" t="n">
+        <v>34.99986674354398</v>
+      </c>
       <c r="O248" t="n">
         <v>27.9314693694032</v>
       </c>
@@ -21278,9 +23501,18 @@
       <c r="J249" t="n">
         <v>0.61</v>
       </c>
+      <c r="K249" t="n">
+        <v>0.5819899060142225</v>
+      </c>
+      <c r="L249" t="n">
+        <v>0.5820282632877321</v>
+      </c>
       <c r="M249" t="n">
         <v>34.8541</v>
       </c>
+      <c r="N249" t="n">
+        <v>35.02164963501765</v>
+      </c>
       <c r="O249" t="n">
         <v>27.95724918487258</v>
       </c>
@@ -21364,9 +23596,18 @@
       <c r="J250" t="n">
         <v>0.3049</v>
       </c>
+      <c r="K250" t="n">
+        <v>0.2685238510033622</v>
+      </c>
+      <c r="L250" t="n">
+        <v>0.268267679236016</v>
+      </c>
       <c r="M250" t="n">
         <v>34.8675</v>
       </c>
+      <c r="N250" t="n">
+        <v>35.0349446622165</v>
+      </c>
       <c r="O250" t="n">
         <v>27.98661964539292</v>
       </c>
@@ -21450,9 +23691,18 @@
       <c r="J251" t="n">
         <v>0.0463</v>
       </c>
+      <c r="K251" t="n">
+        <v>0.001362567645176107</v>
+      </c>
+      <c r="L251" t="n">
+        <v>0.0008415565025053824</v>
+      </c>
       <c r="M251" t="n">
         <v>34.878</v>
       </c>
+      <c r="N251" t="n">
+        <v>35.04550464287298</v>
+      </c>
       <c r="O251" t="n">
         <v>28.00997741516335</v>
       </c>
@@ -21536,9 +23786,18 @@
       <c r="J252" t="n">
         <v>-0.292</v>
       </c>
+      <c r="K252" t="n">
+        <v>-0.362000201882378</v>
+      </c>
+      <c r="L252" t="n">
+        <v>-0.3628187564437204</v>
+      </c>
       <c r="M252" t="n">
         <v>34.9116</v>
       </c>
+      <c r="N252" t="n">
+        <v>35.07983129420841</v>
+      </c>
       <c r="O252" t="n">
         <v>28.0561841536371</v>
       </c>
@@ -21622,9 +23881,18 @@
       <c r="J253" t="n">
         <v>-0.4021</v>
       </c>
+      <c r="K253" t="n">
+        <v>-0.5030746892277704</v>
+      </c>
+      <c r="L253" t="n">
+        <v>-0.5039511498545844</v>
+      </c>
       <c r="M253" t="n">
         <v>34.9431</v>
       </c>
+      <c r="N253" t="n">
+        <v>35.11179912130734</v>
+      </c>
       <c r="O253" t="n">
         <v>28.08867102538693</v>
       </c>
@@ -21708,9 +23976,18 @@
       <c r="J254" t="n">
         <v>-0.3842</v>
       </c>
+      <c r="K254" t="n">
+        <v>-0.5138608929823054</v>
+      </c>
+      <c r="L254" t="n">
+        <v>-0.5147129272935145</v>
+      </c>
       <c r="M254" t="n">
         <v>34.9536</v>
       </c>
+      <c r="N254" t="n">
+        <v>35.12239468919897</v>
+      </c>
       <c r="O254" t="n">
         <v>28.09770939754435</v>
       </c>
@@ -21794,8 +24071,17 @@
       <c r="J255" t="n">
         <v>-0.2931</v>
       </c>
+      <c r="K255" t="n">
+        <v>-0.5041173574457573</v>
+      </c>
+      <c r="L255" t="n">
+        <v>-0.5049349174707894</v>
+      </c>
       <c r="M255" t="n">
         <v>34.959</v>
+      </c>
+      <c r="N255" t="n">
+        <v>35.12843289612477</v>
       </c>
       <c r="O255" t="n">
         <v>28.10210329491997</v>

</xml_diff>